<commit_message>
Dash Hedge IPCA - 2026-04-10
</commit_message>
<xml_diff>
--- a/Dados/Atualizar.xlsx
+++ b/Dados/Atualizar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\livia.jacob\Desktop\Hedge IPCA teste\Projeto-Hedge-IPCA\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DC4E0A-D513-4B11-AF08-DA076ADF3BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D624B7C6-5BF2-491A-B22C-A16FDCC4AE13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-1260" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -18,52 +18,52 @@
     <sheet name="Planilha2" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_ECO_RANGE_ID007ff5be29854ce39e6138063cf998bc" localSheetId="2" hidden="1">Planilha2!$K$4:$K$497</definedName>
-    <definedName name="_ECO_RANGE_ID07302fdece764c078b652f1355f84a96" localSheetId="0" hidden="1">Plan1!$H$4:$H$497</definedName>
-    <definedName name="_ECO_RANGE_ID0da8e0271ec447fa953cbd178dd0e58a" localSheetId="1" hidden="1">Planilha1!$N$4:$N$497</definedName>
-    <definedName name="_ECO_RANGE_ID1cd88e4aa7b843cfad8c1b37d7e9b4b6" localSheetId="0" hidden="1">Plan1!$J$4:$J$497</definedName>
-    <definedName name="_ECO_RANGE_ID261c850c8dc14173940dcdf7f692c4fc" localSheetId="2" hidden="1">Planilha2!$L$4:$L$497</definedName>
-    <definedName name="_ECO_RANGE_ID27b97db650134309895d94a7bbb026bc" localSheetId="2" hidden="1">Planilha2!$G$4:$G$497</definedName>
-    <definedName name="_ECO_RANGE_ID2a56de7d19004fe09a50dd618014af2a" localSheetId="2" hidden="1">Planilha2!$N$4:$N$497</definedName>
-    <definedName name="_ECO_RANGE_ID2bc600552c274a1b9eabf33583033f6c" localSheetId="1" hidden="1">Planilha1!$K$4:$K$497</definedName>
-    <definedName name="_ECO_RANGE_ID37a52560ecd9482b80c24c2951732202" localSheetId="1" hidden="1">Planilha1!$J$4:$J$497</definedName>
-    <definedName name="_ECO_RANGE_ID46651bfa4312428f9c21b3cfb4fb7449" localSheetId="1" hidden="1">Planilha1!$B$3</definedName>
-    <definedName name="_ECO_RANGE_ID4d56951d8cc440d3bbf9b57d867802df" localSheetId="1" hidden="1">Planilha1!$I$4:$I$497</definedName>
-    <definedName name="_ECO_RANGE_ID4ed32a8b5b214cb9ac8829479f78e691" localSheetId="1" hidden="1">Planilha1!$H$4:$H$497</definedName>
-    <definedName name="_ECO_RANGE_ID59dc6b7829474ba385d9f4ffd7358e9c" localSheetId="1" hidden="1">Planilha1!$L$4:$L$497</definedName>
-    <definedName name="_ECO_RANGE_ID5a2a042ba41f43a0b00ec04d5d85a117" localSheetId="1" hidden="1">Planilha1!$A$4:$B$497</definedName>
-    <definedName name="_ECO_RANGE_ID5e23e20ea98a4b65aa4ab1c49f465a94" localSheetId="0" hidden="1">Plan1!$K$4:$K$497</definedName>
-    <definedName name="_ECO_RANGE_ID65ed3e75943148d48b469e4ba6efe977" localSheetId="1" hidden="1">Planilha1!$G$4:$G$497</definedName>
-    <definedName name="_ECO_RANGE_ID674a092cd224453fa610816fcdfe7d72" localSheetId="2" hidden="1">Planilha2!$H$4:$H$497</definedName>
-    <definedName name="_ECO_RANGE_ID67c821f8e1a848edb45e95a970c1304f" localSheetId="2" hidden="1">Planilha2!$J$4:$J$497</definedName>
-    <definedName name="_ECO_RANGE_ID685e9fda394e4ba0962f64c465aeda5c" localSheetId="0" hidden="1">Plan1!$F$4:$F$497</definedName>
-    <definedName name="_ECO_RANGE_ID701dcf9f96404d4893d0e8a826ef9b71" localSheetId="0" hidden="1">Plan1!$C$4:$C$497</definedName>
-    <definedName name="_ECO_RANGE_ID740cae7b20cd4876ae35636ddaad7e74" localSheetId="2" hidden="1">Planilha2!$P$4:$P$497</definedName>
-    <definedName name="_ECO_RANGE_ID747bf1ccb703491ea3cbf477832dcadb" localSheetId="2" hidden="1">Planilha2!$I$4:$I$497</definedName>
-    <definedName name="_ECO_RANGE_ID7532cb0439e246088651a66b70cca5e3" localSheetId="0" hidden="1">Plan1!$L$4:$L$497</definedName>
-    <definedName name="_ECO_RANGE_ID773469f7fde946b6aa45c09ca0102557" localSheetId="0" hidden="1">Plan1!$I$4:$I$497</definedName>
-    <definedName name="_ECO_RANGE_ID789bca61c58441a98710ddf57faa8b4a" localSheetId="1" hidden="1">Planilha1!$E$4:$E$497</definedName>
-    <definedName name="_ECO_RANGE_ID78d93b0a70994e4786b2d2bff275c48f" localSheetId="2" hidden="1">Planilha2!$O$4:$O$497</definedName>
-    <definedName name="_ECO_RANGE_ID8a52508c480745ad91a88002c334d868" localSheetId="1" hidden="1">Planilha1!$F$4:$F$497</definedName>
-    <definedName name="_ECO_RANGE_ID8b138e5047a74cc690b6c3cf8eb3cc4c" localSheetId="0" hidden="1">Plan1!$D$4:$D$497</definedName>
-    <definedName name="_ECO_RANGE_ID91456274deec4304a9608205f443d6b8" localSheetId="1" hidden="1">Planilha1!$D$4:$D$497</definedName>
-    <definedName name="_ECO_RANGE_ID93af163ef3bd4160a7c90f285bd52a88" localSheetId="0" hidden="1">Plan1!$B$3</definedName>
-    <definedName name="_ECO_RANGE_ID9a781331a79c483fae1091ac8c64739a" localSheetId="0" hidden="1">Plan1!$M$4:$M$497</definedName>
-    <definedName name="_ECO_RANGE_ID9d5700d030474c68beae95569184d6c0" localSheetId="0" hidden="1">Plan1!$N$4:$N$497</definedName>
-    <definedName name="_ECO_RANGE_IDa572e51d4cb6403f8f092c3a7a113057" localSheetId="2" hidden="1">Planilha2!$F$4:$F$497</definedName>
-    <definedName name="_ECO_RANGE_IDa5f174076b4b490eb74b349130b7916b" localSheetId="1" hidden="1">Planilha1!$M$4:$M$497</definedName>
-    <definedName name="_ECO_RANGE_IDa7b486806fc94c42b8be3953a42ffb4e" localSheetId="2" hidden="1">Planilha2!$D$4:$D$497</definedName>
-    <definedName name="_ECO_RANGE_IDac939ff5f968468b8b8b251944210ce7" localSheetId="2" hidden="1">Planilha2!$E$4:$E$497</definedName>
-    <definedName name="_ECO_RANGE_IDae4bc00a0e224e2b99d6f10c33759142" localSheetId="2" hidden="1">Planilha2!$B$3</definedName>
-    <definedName name="_ECO_RANGE_IDbdd74e8bad7d49708531ba6195a2ad4b" localSheetId="1" hidden="1">Planilha1!$O$4:$O$497</definedName>
-    <definedName name="_ECO_RANGE_IDbf7b97c74b9b47acb76d52e6fa317f6d" localSheetId="2" hidden="1">Planilha2!$C$4:$C$497</definedName>
-    <definedName name="_ECO_RANGE_IDc01cade5dccd4ba3adef5dc4bb6ae908" localSheetId="0" hidden="1">Plan1!$O$4:$O$497</definedName>
-    <definedName name="_ECO_RANGE_IDce764c48b07044d2bb04a0ad806fbf6a" localSheetId="1" hidden="1">Planilha1!$C$4:$C$497</definedName>
-    <definedName name="_ECO_RANGE_IDd114bec021ff44478f103810bdc597d0" localSheetId="0" hidden="1">Plan1!$G$4:$G$497</definedName>
-    <definedName name="_ECO_RANGE_IDe2287078621a4419a7de27732e56d76a" localSheetId="2" hidden="1">Planilha2!$A$4:$B$497</definedName>
-    <definedName name="_ECO_RANGE_IDefbaebce234a43e8bf2ae164fa9d3de5" localSheetId="0" hidden="1">Plan1!$A$4:$B$497</definedName>
-    <definedName name="_ECO_RANGE_IDf0272171b29b4c0094838678829c76c5" localSheetId="0" hidden="1">Plan1!$E$4:$E$497</definedName>
-    <definedName name="_ECO_RANGE_IDf57c290189924f458f4c17cae4d3e1f9" localSheetId="2" hidden="1">Planilha2!$M$4:$M$497</definedName>
+    <definedName name="_ECO_RANGE_ID00e76574b0624b3f80d0e29bd2420585" localSheetId="2" hidden="1">Planilha2!$I$4:$I$511</definedName>
+    <definedName name="_ECO_RANGE_ID0ca2184d708a4271baf003d9a1c716da" localSheetId="1" hidden="1">Planilha1!$B$3</definedName>
+    <definedName name="_ECO_RANGE_ID1c21957cb5054573a1d238750a58a67e" localSheetId="1" hidden="1">Planilha1!$A$4:$B$511</definedName>
+    <definedName name="_ECO_RANGE_ID1d28d9a8f21f494e8ce2ea4d34ae2699" localSheetId="1" hidden="1">Planilha1!$K$4:$K$511</definedName>
+    <definedName name="_ECO_RANGE_ID1e171e8255724b69b1039f752a0c6357" localSheetId="2" hidden="1">Planilha2!$P$4:$P$511</definedName>
+    <definedName name="_ECO_RANGE_ID1f847766b5984ccf829f829bbee3c277" localSheetId="2" hidden="1">Planilha2!$J$4:$J$511</definedName>
+    <definedName name="_ECO_RANGE_ID2263af481ec0463180d115747aa43df9" localSheetId="1" hidden="1">Planilha1!$J$4:$J$511</definedName>
+    <definedName name="_ECO_RANGE_ID232ebef712f94d0b81b56c536489891c" localSheetId="0" hidden="1">Plan1!$F$4:$F$511</definedName>
+    <definedName name="_ECO_RANGE_ID2456f6dbaf9a46f9a7a8da48def4aaa5" localSheetId="0" hidden="1">Plan1!$G$4:$G$511</definedName>
+    <definedName name="_ECO_RANGE_ID254e87af413c4cb986cdc16f2c5dffae" localSheetId="2" hidden="1">Planilha2!$O$4:$O$511</definedName>
+    <definedName name="_ECO_RANGE_ID2857e1655bd94ecda14895a570f07374" localSheetId="2" hidden="1">Planilha2!$M$4:$M$511</definedName>
+    <definedName name="_ECO_RANGE_ID2bf3f203bdd04613a6363ea76bf46229" localSheetId="2" hidden="1">Planilha2!$C$4:$C$511</definedName>
+    <definedName name="_ECO_RANGE_ID3937a644b00e41c18364273ec40793bc" localSheetId="0" hidden="1">Plan1!$L$4:$L$511</definedName>
+    <definedName name="_ECO_RANGE_ID3b23869efc324a4abe9ccfbb4b298e60" localSheetId="1" hidden="1">Planilha1!$L$4:$L$511</definedName>
+    <definedName name="_ECO_RANGE_ID3b743473a33142c6b9458acec2a37261" localSheetId="1" hidden="1">Planilha1!$E$4:$E$511</definedName>
+    <definedName name="_ECO_RANGE_ID473fe07ab4704df8bffef6945131b806" localSheetId="0" hidden="1">Plan1!$J$4:$J$511</definedName>
+    <definedName name="_ECO_RANGE_ID47b5330b869b40ebb1412c1f212c5686" localSheetId="0" hidden="1">Plan1!$I$4:$I$511</definedName>
+    <definedName name="_ECO_RANGE_ID54af0d7ac46f4f83a05fbe311eb66f59" localSheetId="0" hidden="1">Plan1!$E$4:$E$511</definedName>
+    <definedName name="_ECO_RANGE_ID5b747179ed9b40c090504187252e6c12" localSheetId="2" hidden="1">Planilha2!$N$4:$N$511</definedName>
+    <definedName name="_ECO_RANGE_ID5e9abdc0d24d42d582f711ff881e0cc7" localSheetId="2" hidden="1">Planilha2!$H$4:$H$511</definedName>
+    <definedName name="_ECO_RANGE_ID6b39f817d71a492b8d4a3485ec2533e8" localSheetId="0" hidden="1">Plan1!$C$4:$C$511</definedName>
+    <definedName name="_ECO_RANGE_ID6d5830ca54f24720bb7fa7ab018c5b91" localSheetId="2" hidden="1">Planilha2!$B$3</definedName>
+    <definedName name="_ECO_RANGE_ID77ac73d043e24720b080ca54f777d98d" localSheetId="1" hidden="1">Planilha1!$F$4:$F$511</definedName>
+    <definedName name="_ECO_RANGE_ID7cfb044391844e06ba8843b0d19da22f" localSheetId="2" hidden="1">Planilha2!$K$4:$K$511</definedName>
+    <definedName name="_ECO_RANGE_ID7d562063ae1843d699e06abbad50c403" localSheetId="0" hidden="1">Plan1!$K$4:$K$511</definedName>
+    <definedName name="_ECO_RANGE_ID7d8b621180af48ebbbc3c410be289395" localSheetId="1" hidden="1">Planilha1!$D$4:$D$511</definedName>
+    <definedName name="_ECO_RANGE_ID7daf296a8e4c4c26a5d2bde7a75c235e" localSheetId="0" hidden="1">Plan1!$M$4:$M$511</definedName>
+    <definedName name="_ECO_RANGE_ID9aabd0f32504463a96b4226636091fb2" localSheetId="2" hidden="1">Planilha2!$A$4:$B$511</definedName>
+    <definedName name="_ECO_RANGE_ID9d45bf1d2cab443db565260ba3806640" localSheetId="0" hidden="1">Plan1!$D$4:$D$511</definedName>
+    <definedName name="_ECO_RANGE_ID9ecd5d7c51554ce6ba1480d8c3eee854" localSheetId="2" hidden="1">Planilha2!$E$4:$E$511</definedName>
+    <definedName name="_ECO_RANGE_IDa12df9e429f44a729e21711af60e42e8" localSheetId="0" hidden="1">Plan1!$N$4:$N$511</definedName>
+    <definedName name="_ECO_RANGE_IDa887542f3b7846f2afb9502f13811566" localSheetId="0" hidden="1">Plan1!$O$4:$O$511</definedName>
+    <definedName name="_ECO_RANGE_IDab70849247ca481896605025d66a800b" localSheetId="1" hidden="1">Planilha1!$N$4:$N$511</definedName>
+    <definedName name="_ECO_RANGE_IDad723ae37f574a4197d1df789db1c529" localSheetId="1" hidden="1">Planilha1!$O$4:$O$511</definedName>
+    <definedName name="_ECO_RANGE_IDb804cfc80e9043d9af304e043a31d260" localSheetId="0" hidden="1">Plan1!$B$3</definedName>
+    <definedName name="_ECO_RANGE_IDb96a28ff555545e4aaaebc6c701a168d" localSheetId="2" hidden="1">Planilha2!$F$4:$F$511</definedName>
+    <definedName name="_ECO_RANGE_IDc7b478ef50304093bb8e5bf40a17c94c" localSheetId="2" hidden="1">Planilha2!$G$4:$G$511</definedName>
+    <definedName name="_ECO_RANGE_IDcdd812b56b634f0e819953c5e571c66e" localSheetId="1" hidden="1">Planilha1!$I$4:$I$511</definedName>
+    <definedName name="_ECO_RANGE_IDd061a8b7d8714484b222e53980f0e91a" localSheetId="1" hidden="1">Planilha1!$H$4:$H$511</definedName>
+    <definedName name="_ECO_RANGE_IDd5577f4583464d118628ec8007f31230" localSheetId="1" hidden="1">Planilha1!$G$4:$G$511</definedName>
+    <definedName name="_ECO_RANGE_IDda57c28fb56c4536913e96798d0e8fb6" localSheetId="0" hidden="1">Plan1!$H$4:$H$511</definedName>
+    <definedName name="_ECO_RANGE_IDe31d00163de0498c9ac7cb0a33c5a73f" localSheetId="0" hidden="1">Plan1!$A$4:$B$511</definedName>
+    <definedName name="_ECO_RANGE_IDe3fe4b7a712d41c48173b5ff41e2769e" localSheetId="1" hidden="1">Planilha1!$C$4:$C$511</definedName>
+    <definedName name="_ECO_RANGE_IDe9544339a6694282ab37faa936de2ab2" localSheetId="2" hidden="1">Planilha2!$L$4:$L$511</definedName>
+    <definedName name="_ECO_RANGE_IDf58054575add4fd2a046a2c25a6473e7" localSheetId="2" hidden="1">Planilha2!$D$4:$D$511</definedName>
+    <definedName name="_ECO_RANGE_IDf7a9036fd4df40249838f740cd819492" localSheetId="1" hidden="1">Planilha1!$M$4:$M$511</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -284,306 +284,300 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
       <tp>
         <v>3</v>
         <stp/>
-        <stp>8912f892-5923-477a-89f5-f7cb8ef3d9d1</stp>
-        <tr r="L3" s="3"/>
+        <stp>651e0012-4377-47a7-bd8e-2053c1351fc1</stp>
+        <tr r="O3" s="2"/>
       </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
       <tp>
         <v>3</v>
         <stp/>
-        <stp>a845e5f7-eec2-4247-b2fe-327b3680de35</stp>
-        <tr r="J3" s="1"/>
+        <stp>5c284fe6-32ce-4540-9e0b-b8dfeb18055b</stp>
+        <tr r="I3" s="3"/>
       </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
       <tp>
         <v>3</v>
         <stp/>
-        <stp>89ee2c17-f8ee-4757-b5d5-ef6c1595bb56</stp>
+        <stp>0fae79ac-b820-4bef-bbcd-e60ae439ec0a</stp>
+        <tr r="F3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>b141a3b4-55d4-4bde-a394-c076c3fbe012</stp>
+        <tr r="H3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>8f5fba8f-79ad-4e6b-999a-44c71b05de57</stp>
+        <tr r="C3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a2251b01-aedc-4289-aa18-14afd4015a39</stp>
+        <tr r="H3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>83bcbf2c-ab75-4fde-b420-08aa99a7b80a</stp>
+        <tr r="F3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>34ed34ea-4bea-411b-806a-992e1275463b</stp>
+        <tr r="E3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>aa60246a-c683-4068-b6ff-f4a05b633be6</stp>
         <tr r="E3" s="2"/>
       </tp>
       <tp>
         <v>3</v>
         <stp/>
-        <stp>98b3e0c8-ae18-4947-98a2-cd1f0d191a3e</stp>
-        <tr r="N3" s="2"/>
+        <stp>3b76ab7a-d3ac-4c52-87e5-b8f44a56d691</stp>
+        <tr r="L3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>612ef0ab-c5a9-4644-8c16-bea17d5da981</stp>
+        <tr r="A3" s="3"/>
       </tp>
       <tp>
         <v>3</v>
         <stp/>
-        <stp>5545e99f-e3b3-425c-acd3-fa8bfdc0459b</stp>
-        <tr r="F3" s="1"/>
+        <stp>5a276a4e-a38b-4ea7-8a95-5ca0fe80c6c3</stp>
+        <tr r="F3" s="2"/>
       </tp>
       <tp>
         <v>3</v>
         <stp/>
-        <stp>39016a73-7216-4e37-81ab-7fb7bae3bca4</stp>
-        <tr r="I3" s="3"/>
+        <stp>6ba51716-09d3-402a-9998-daf254bb370f</stp>
+        <tr r="C3" s="1"/>
       </tp>
     </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
       <tp>
         <v>3</v>
         <stp/>
-        <stp>ed30af17-921b-43b3-acf3-66bb8f34fc5a</stp>
+        <stp>0ce85a8e-5771-4ebf-83a3-49eec1a13fd0</stp>
+        <tr r="K3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>40fb259b-7203-4902-ae09-e0e7283e1fa0</stp>
+        <tr r="K3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a06e5785-eae8-4cd1-8428-0aaedbadc337</stp>
+        <tr r="G3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>6bf6d21a-a716-4e10-bd45-b46aea434136</stp>
+        <tr r="M3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>2ac33508-667b-42d5-ac3a-16c530cf73a7</stp>
+        <tr r="D3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>9a829019-f63f-4980-a213-d1b97ef15204</stp>
+        <tr r="D3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>4a14c25a-c931-410f-ab82-7313393ee44b</stp>
+        <tr r="M3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>09141432-6a45-4e29-91c2-d2809d270ded</stp>
+        <tr r="C3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>cf48377e-438f-4f4d-b3d9-3aa155539b53</stp>
+        <tr r="A3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>6aa58b9c-5de2-4307-ac19-61a0350c5ffd</stp>
+        <tr r="L3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>71862d1f-1374-431a-8907-d2c83f1c93d7</stp>
+        <tr r="M3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>1e0f62dc-a1b4-4ce5-a9ac-efb12ba313ba</stp>
+        <tr r="H3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>bb586066-c948-457d-bbdc-5a93e06ec477</stp>
+        <tr r="N3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>e998bcf1-d070-44b4-bbd2-f812f46204ac</stp>
+        <tr r="N3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>f2cd3e29-b279-4188-936c-10caa4e5b67f</stp>
+        <tr r="K3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a9db0880-6629-4e1d-848d-c167f5cb4fd7</stp>
+        <tr r="G3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>7c8665e3-0701-46db-a91d-76e6635ef941</stp>
+        <tr r="D3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>2997b43d-a6ac-4fcc-a4ff-a3d4ec9a423e</stp>
+        <tr r="L3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>f1fb2c7a-646a-439c-ad4d-e904c23c53a4</stp>
+        <tr r="A3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>e85303c7-4450-4411-87a5-6f5b6f0b6eb0</stp>
+        <tr r="E3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>4c0b1ccd-b2cd-4ccd-a922-2a4f1a2c194e</stp>
+        <tr r="J3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>97aaf7e5-f754-43e9-94e9-62ad665aa1a0</stp>
+        <tr r="N3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>92bb70ff-4e9e-4457-9ad7-924b8e6e60ca</stp>
+        <tr r="G3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>ea97e4ec-9e47-43be-9392-5e57d3e4cdbb</stp>
+        <tr r="I3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>c62f33e1-bb3c-40e5-a564-6ef9fe0c6aed</stp>
+        <tr r="O3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>1f63dc19-d7ea-4680-840b-1f9c8cec5a77</stp>
         <tr r="O3" s="1"/>
       </tp>
       <tp>
         <v>3</v>
         <stp/>
-        <stp>93cfc8de-e98c-4e6f-9040-043ac3d34f10</stp>
-        <tr r="N3" s="3"/>
+        <stp>99089bdc-7689-4349-b886-e8fecde4044b</stp>
+        <tr r="J3" s="3"/>
       </tp>
     </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
       <tp>
         <v>3</v>
         <stp/>
-        <stp>f7d30019-189b-4eb0-806f-d76ff7ff2c90</stp>
-        <tr r="D3" s="3"/>
+        <stp>7d8fb1cc-613d-4f1e-b66b-c2d8771ae156</stp>
+        <tr r="I3" s="1"/>
       </tp>
+    </main>
+    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
       <tp>
         <v>3</v>
         <stp/>
-        <stp>1c8e5fb0-84d2-467c-9f62-7f36be86088d</stp>
-        <tr r="J3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>f8a95550-4709-4634-a586-d56ead0b66ed</stp>
-        <tr r="D3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>2234423e-ad40-4b4e-b025-95c4d308fb9a</stp>
-        <tr r="C3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>5c867bbb-8312-4d0e-88c5-080a312ddd73</stp>
-        <tr r="C3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>b1e19b20-2136-416e-b10a-5b28fb7eae7d</stp>
-        <tr r="F3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>9f4ce07f-6364-41db-a2dd-d3de5e5fba2a</stp>
-        <tr r="O3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>3268f807-b9b0-402b-8b80-bbe47553d44e</stp>
-        <tr r="M3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>22c748b6-9b24-45e2-80ce-fe3bf1c22a6f</stp>
-        <tr r="A3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>7076b515-6122-4df2-af2f-05e06ee0248f</stp>
-        <tr r="G3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>b27012d5-afe4-4266-ae5c-5ee09338db19</stp>
-        <tr r="K3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>ee86f366-0ef5-419f-947f-c253f1dc6be1</stp>
-        <tr r="O3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>066bb603-66d3-475a-8525-346343c8c49d</stp>
-        <tr r="I3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>a318421f-926f-4cc8-8b50-6e41630b3724</stp>
-        <tr r="E3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>5d604963-c66e-4f08-b069-6ddef209e20e</stp>
-        <tr r="M3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>9a142539-22c8-4dcc-8765-bd15eee85958</stp>
-        <tr r="G3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>a861d6f8-b206-4d62-b0ef-6b8ba5849e14</stp>
-        <tr r="H3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>8c25453d-f0e6-40ba-988e-507f2bb903ed</stp>
-        <tr r="G3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>065765c2-977c-49c3-b8ce-2ae36e21da25</stp>
-        <tr r="H3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>a120b285-89d0-421a-83dc-17d294a95391</stp>
-        <tr r="N3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>de38956b-4117-4d94-bb6e-3fa45856758d</stp>
-        <tr r="L3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>b7979dea-1ea5-4e2e-9ad1-54791b1c4803</stp>
-        <tr r="D3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>7690881f-6e54-4862-a207-be51f9155e9c</stp>
-        <tr r="L3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>5eae153c-71b5-44f9-8149-ea6ad07de875</stp>
-        <tr r="K3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>8f550fe8-c489-410c-af1b-ddb4636eedfc</stp>
-        <tr r="M3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>eb6b404b-b8ed-4235-802d-4330d1fdd707</stp>
+        <stp>4118678b-6a94-4506-931e-9495ac877f90</stp>
         <tr r="P3" s="3"/>
       </tp>
       <tp>
         <v>3</v>
         <stp/>
-        <stp>48ca3e95-ed67-4780-83ab-1945b46f4f41</stp>
-        <tr r="A3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>5f22f515-a6f4-46e4-b82f-0d6422432c93</stp>
-        <tr r="K3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>1de34262-e77c-4ae9-b1cc-c4750887ce91</stp>
-        <tr r="I3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>444a1796-3cb6-4155-9b4c-3b506e1b81ce</stp>
-        <tr r="H3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>1284bb87-26df-4515-94f6-7a958c63f4da</stp>
-        <tr r="J3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>3fb2f918-e112-44a8-82ce-f53754750f98</stp>
-        <tr r="E3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>8947e605-d576-4207-a84e-d0e61dd509c8</stp>
-        <tr r="C3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_7697892fda974de08ff0ddcf1f2c69ca">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>0b115674-2b99-4482-bb77-b04e94942bb7</stp>
-        <tr r="F3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>63053cab-645d-49ca-a903-2ccfe6ddef30</stp>
-        <tr r="A3" s="3"/>
+        <stp>3fd1c9b3-4cf8-4aab-9f4b-39c2877875c2</stp>
+        <tr r="J3" s="2"/>
       </tp>
     </main>
   </volType>
@@ -853,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O497"/>
+  <dimension ref="A1:O511"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -22870,6 +22864,583 @@
         <v>7.2374000000000001</v>
       </c>
     </row>
+    <row r="498" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A498" s="1">
+        <v>46104</v>
+      </c>
+      <c r="C498">
+        <v>9.1445000000000007</v>
+      </c>
+      <c r="D498">
+        <v>8.1598000000000006</v>
+      </c>
+      <c r="E498">
+        <v>8.0203000000000007</v>
+      </c>
+      <c r="F498">
+        <v>7.9005999999999998</v>
+      </c>
+      <c r="G498">
+        <v>7.9363000000000001</v>
+      </c>
+      <c r="H498">
+        <v>7.8315000000000001</v>
+      </c>
+      <c r="I498">
+        <v>7.8231000000000002</v>
+      </c>
+      <c r="J498">
+        <v>7.6208999999999998</v>
+      </c>
+      <c r="K498">
+        <v>7.3489000000000004</v>
+      </c>
+      <c r="L498">
+        <v>7.2766000000000002</v>
+      </c>
+      <c r="M498">
+        <v>7.2343000000000002</v>
+      </c>
+      <c r="N498">
+        <v>7.1993999999999998</v>
+      </c>
+      <c r="O498">
+        <v>7.2313000000000001</v>
+      </c>
+    </row>
+    <row r="499" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A499" s="1">
+        <v>46105</v>
+      </c>
+      <c r="C499">
+        <v>9.1292000000000009</v>
+      </c>
+      <c r="D499">
+        <v>8.1830999999999996</v>
+      </c>
+      <c r="E499">
+        <v>8.06</v>
+      </c>
+      <c r="F499">
+        <v>7.9615999999999998</v>
+      </c>
+      <c r="G499">
+        <v>7.9908999999999999</v>
+      </c>
+      <c r="H499">
+        <v>7.8895999999999997</v>
+      </c>
+      <c r="I499">
+        <v>7.87</v>
+      </c>
+      <c r="J499">
+        <v>7.6576000000000004</v>
+      </c>
+      <c r="K499">
+        <v>7.3921000000000001</v>
+      </c>
+      <c r="L499">
+        <v>7.3186999999999998</v>
+      </c>
+      <c r="M499">
+        <v>7.2729999999999997</v>
+      </c>
+      <c r="N499">
+        <v>7.2489999999999997</v>
+      </c>
+      <c r="O499">
+        <v>7.2632000000000003</v>
+      </c>
+    </row>
+    <row r="500" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A500" s="1">
+        <v>46106</v>
+      </c>
+      <c r="C500">
+        <v>9.1801999999999992</v>
+      </c>
+      <c r="D500">
+        <v>8.15</v>
+      </c>
+      <c r="E500">
+        <v>8.02</v>
+      </c>
+      <c r="F500">
+        <v>7.9291999999999998</v>
+      </c>
+      <c r="G500">
+        <v>7.96</v>
+      </c>
+      <c r="H500">
+        <v>7.8451000000000004</v>
+      </c>
+      <c r="I500">
+        <v>7.8292000000000002</v>
+      </c>
+      <c r="J500">
+        <v>7.6367000000000003</v>
+      </c>
+      <c r="K500">
+        <v>7.39</v>
+      </c>
+      <c r="L500">
+        <v>7.3010999999999999</v>
+      </c>
+      <c r="M500">
+        <v>7.2625000000000002</v>
+      </c>
+      <c r="N500">
+        <v>7.2561</v>
+      </c>
+      <c r="O500">
+        <v>7.2587000000000002</v>
+      </c>
+    </row>
+    <row r="501" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A501" s="1">
+        <v>46107</v>
+      </c>
+      <c r="C501">
+        <v>8.7395999999999994</v>
+      </c>
+      <c r="D501">
+        <v>8.1807999999999996</v>
+      </c>
+      <c r="E501">
+        <v>8.1141000000000005</v>
+      </c>
+      <c r="F501">
+        <v>8.0061</v>
+      </c>
+      <c r="G501">
+        <v>8.0302000000000007</v>
+      </c>
+      <c r="H501">
+        <v>7.9233000000000002</v>
+      </c>
+      <c r="I501">
+        <v>7.9039999999999999</v>
+      </c>
+      <c r="J501">
+        <v>7.6976000000000004</v>
+      </c>
+      <c r="K501">
+        <v>7.4454000000000002</v>
+      </c>
+      <c r="L501">
+        <v>7.3593000000000002</v>
+      </c>
+      <c r="M501">
+        <v>7.3140999999999998</v>
+      </c>
+      <c r="N501">
+        <v>7.3080999999999996</v>
+      </c>
+      <c r="O501">
+        <v>7.3082000000000003</v>
+      </c>
+    </row>
+    <row r="502" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A502" s="1">
+        <v>46108</v>
+      </c>
+      <c r="C502">
+        <v>9.0396000000000001</v>
+      </c>
+      <c r="D502">
+        <v>8.2634000000000007</v>
+      </c>
+      <c r="E502">
+        <v>8.1356999999999999</v>
+      </c>
+      <c r="F502">
+        <v>8.02</v>
+      </c>
+      <c r="G502">
+        <v>8.0434000000000001</v>
+      </c>
+      <c r="H502">
+        <v>7.94</v>
+      </c>
+      <c r="I502">
+        <v>7.9241000000000001</v>
+      </c>
+      <c r="J502">
+        <v>7.6925999999999997</v>
+      </c>
+      <c r="K502">
+        <v>7.4245999999999999</v>
+      </c>
+      <c r="L502">
+        <v>7.3525999999999998</v>
+      </c>
+      <c r="M502">
+        <v>7.3151999999999999</v>
+      </c>
+      <c r="N502">
+        <v>7.31</v>
+      </c>
+      <c r="O502">
+        <v>7.31</v>
+      </c>
+    </row>
+    <row r="503" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A503" s="1">
+        <v>46111</v>
+      </c>
+      <c r="C503">
+        <v>8.9133999999999993</v>
+      </c>
+      <c r="D503">
+        <v>8.0488999999999997</v>
+      </c>
+      <c r="E503">
+        <v>8.01</v>
+      </c>
+      <c r="F503">
+        <v>7.9364999999999997</v>
+      </c>
+      <c r="G503">
+        <v>7.97</v>
+      </c>
+      <c r="H503">
+        <v>7.8845999999999998</v>
+      </c>
+      <c r="I503">
+        <v>7.8673999999999999</v>
+      </c>
+      <c r="J503">
+        <v>7.6772</v>
+      </c>
+      <c r="K503">
+        <v>7.4436999999999998</v>
+      </c>
+      <c r="L503">
+        <v>7.36</v>
+      </c>
+      <c r="M503">
+        <v>7.31</v>
+      </c>
+      <c r="N503">
+        <v>7.3094999999999999</v>
+      </c>
+      <c r="O503">
+        <v>7.2972000000000001</v>
+      </c>
+    </row>
+    <row r="504" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A504" s="1">
+        <v>46112</v>
+      </c>
+      <c r="C504">
+        <v>8.9270999999999994</v>
+      </c>
+      <c r="D504">
+        <v>7.9272</v>
+      </c>
+      <c r="E504">
+        <v>7.8425000000000002</v>
+      </c>
+      <c r="F504">
+        <v>7.7878999999999996</v>
+      </c>
+      <c r="G504">
+        <v>7.8093000000000004</v>
+      </c>
+      <c r="H504">
+        <v>7.7340999999999998</v>
+      </c>
+      <c r="I504">
+        <v>7.7236000000000002</v>
+      </c>
+      <c r="J504">
+        <v>7.5622999999999996</v>
+      </c>
+      <c r="K504">
+        <v>7.3960999999999997</v>
+      </c>
+      <c r="L504">
+        <v>7.2908999999999997</v>
+      </c>
+      <c r="M504">
+        <v>7.2432999999999996</v>
+      </c>
+      <c r="N504">
+        <v>7.2388000000000003</v>
+      </c>
+      <c r="O504">
+        <v>7.22</v>
+      </c>
+    </row>
+    <row r="505" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A505" s="1">
+        <v>46113</v>
+      </c>
+      <c r="C505">
+        <v>8.8130000000000006</v>
+      </c>
+      <c r="D505">
+        <v>7.87</v>
+      </c>
+      <c r="E505">
+        <v>7.7949999999999999</v>
+      </c>
+      <c r="F505">
+        <v>7.7534000000000001</v>
+      </c>
+      <c r="G505">
+        <v>7.7805999999999997</v>
+      </c>
+      <c r="H505">
+        <v>7.7</v>
+      </c>
+      <c r="I505">
+        <v>7.69</v>
+      </c>
+      <c r="J505">
+        <v>7.5418000000000003</v>
+      </c>
+      <c r="K505">
+        <v>7.3708</v>
+      </c>
+      <c r="L505">
+        <v>7.2728000000000002</v>
+      </c>
+      <c r="M505">
+        <v>7.2118000000000002</v>
+      </c>
+      <c r="N505">
+        <v>7.1970999999999998</v>
+      </c>
+      <c r="O505">
+        <v>7.1897000000000002</v>
+      </c>
+    </row>
+    <row r="506" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A506" s="1">
+        <v>46114</v>
+      </c>
+      <c r="C506">
+        <v>8.6003000000000007</v>
+      </c>
+      <c r="D506">
+        <v>7.82</v>
+      </c>
+      <c r="E506">
+        <v>7.8030999999999997</v>
+      </c>
+      <c r="F506">
+        <v>7.7763</v>
+      </c>
+      <c r="G506">
+        <v>7.82</v>
+      </c>
+      <c r="H506">
+        <v>7.7398999999999996</v>
+      </c>
+      <c r="I506">
+        <v>7.7260999999999997</v>
+      </c>
+      <c r="J506">
+        <v>7.5679999999999996</v>
+      </c>
+      <c r="K506">
+        <v>7.3834</v>
+      </c>
+      <c r="L506">
+        <v>7.2545999999999999</v>
+      </c>
+      <c r="M506">
+        <v>7.2119</v>
+      </c>
+      <c r="N506">
+        <v>7.1936999999999998</v>
+      </c>
+      <c r="O506">
+        <v>7.18</v>
+      </c>
+    </row>
+    <row r="507" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A507" s="1">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="508" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A508" s="1">
+        <v>46118</v>
+      </c>
+      <c r="C508">
+        <v>8.6837</v>
+      </c>
+      <c r="D508">
+        <v>7.8764000000000003</v>
+      </c>
+      <c r="E508">
+        <v>7.8623000000000003</v>
+      </c>
+      <c r="F508">
+        <v>7.8170000000000002</v>
+      </c>
+      <c r="G508">
+        <v>7.8400999999999996</v>
+      </c>
+      <c r="H508">
+        <v>7.7426000000000004</v>
+      </c>
+      <c r="I508">
+        <v>7.7233000000000001</v>
+      </c>
+      <c r="J508">
+        <v>7.5731000000000002</v>
+      </c>
+      <c r="K508">
+        <v>7.3791000000000002</v>
+      </c>
+      <c r="L508">
+        <v>7.2337999999999996</v>
+      </c>
+      <c r="M508">
+        <v>7.1760000000000002</v>
+      </c>
+      <c r="N508">
+        <v>7.15</v>
+      </c>
+      <c r="O508">
+        <v>7.1497999999999999</v>
+      </c>
+    </row>
+    <row r="509" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A509" s="1">
+        <v>46119</v>
+      </c>
+      <c r="C509">
+        <v>8.6088000000000005</v>
+      </c>
+      <c r="D509">
+        <v>7.8829000000000002</v>
+      </c>
+      <c r="E509">
+        <v>7.8837999999999999</v>
+      </c>
+      <c r="F509">
+        <v>7.85</v>
+      </c>
+      <c r="G509">
+        <v>7.8845999999999998</v>
+      </c>
+      <c r="H509">
+        <v>7.7641</v>
+      </c>
+      <c r="I509">
+        <v>7.7478999999999996</v>
+      </c>
+      <c r="J509">
+        <v>7.5978000000000003</v>
+      </c>
+      <c r="K509">
+        <v>7.3757000000000001</v>
+      </c>
+      <c r="L509">
+        <v>7.24</v>
+      </c>
+      <c r="M509">
+        <v>7.1826999999999996</v>
+      </c>
+      <c r="N509">
+        <v>7.16</v>
+      </c>
+      <c r="O509">
+        <v>7.1539999999999999</v>
+      </c>
+    </row>
+    <row r="510" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A510" s="1">
+        <v>46120</v>
+      </c>
+      <c r="C510">
+        <v>8.8684999999999992</v>
+      </c>
+      <c r="D510">
+        <v>7.8666999999999998</v>
+      </c>
+      <c r="E510">
+        <v>7.75</v>
+      </c>
+      <c r="F510">
+        <v>7.6932999999999998</v>
+      </c>
+      <c r="G510">
+        <v>7.7</v>
+      </c>
+      <c r="H510">
+        <v>7.6266999999999996</v>
+      </c>
+      <c r="I510">
+        <v>7.6127000000000002</v>
+      </c>
+      <c r="J510">
+        <v>7.4897999999999998</v>
+      </c>
+      <c r="K510">
+        <v>7.2897999999999996</v>
+      </c>
+      <c r="L510">
+        <v>7.1669999999999998</v>
+      </c>
+      <c r="M510">
+        <v>7.1121999999999996</v>
+      </c>
+      <c r="N510">
+        <v>7.0918999999999999</v>
+      </c>
+      <c r="O510">
+        <v>7.0788000000000002</v>
+      </c>
+    </row>
+    <row r="511" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A511" s="1">
+        <v>46121</v>
+      </c>
+      <c r="C511">
+        <v>8.7730999999999995</v>
+      </c>
+      <c r="D511">
+        <v>7.8472999999999997</v>
+      </c>
+      <c r="E511">
+        <v>7.7061000000000002</v>
+      </c>
+      <c r="F511">
+        <v>7.6445999999999996</v>
+      </c>
+      <c r="G511">
+        <v>7.6829000000000001</v>
+      </c>
+      <c r="H511">
+        <v>7.62</v>
+      </c>
+      <c r="I511">
+        <v>7.6</v>
+      </c>
+      <c r="J511">
+        <v>7.47</v>
+      </c>
+      <c r="K511">
+        <v>7.2668999999999997</v>
+      </c>
+      <c r="L511">
+        <v>7.15</v>
+      </c>
+      <c r="M511">
+        <v>7.0934999999999997</v>
+      </c>
+      <c r="N511">
+        <v>7.0673000000000004</v>
+      </c>
+      <c r="O511">
+        <v>7.0507999999999997</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -22877,7 +23448,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2426C424-F8DA-489F-86D1-16CF91ECBA06}">
-  <dimension ref="A1:O497"/>
+  <dimension ref="A1:O511"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -44894,6 +45465,583 @@
         <v>3973.7832149999999</v>
       </c>
     </row>
+    <row r="498" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A498" s="1">
+        <v>46104</v>
+      </c>
+      <c r="C498">
+        <v>4608.3552559999998</v>
+      </c>
+      <c r="D498">
+        <v>4632.0997950000001</v>
+      </c>
+      <c r="E498">
+        <v>4473.1476730000004</v>
+      </c>
+      <c r="F498">
+        <v>4507.739971</v>
+      </c>
+      <c r="G498">
+        <v>4355.8667070000001</v>
+      </c>
+      <c r="H498">
+        <v>4264.5693700000002</v>
+      </c>
+      <c r="I498">
+        <v>4300.4735979999996</v>
+      </c>
+      <c r="J498">
+        <v>4271.4952469999998</v>
+      </c>
+      <c r="K498">
+        <v>4142.9446639999996</v>
+      </c>
+      <c r="L498">
+        <v>4159.2116669999996</v>
+      </c>
+      <c r="M498">
+        <v>4046.7704709999998</v>
+      </c>
+      <c r="N498">
+        <v>4094.004582</v>
+      </c>
+      <c r="O498">
+        <v>3978.5083970000001</v>
+      </c>
+    </row>
+    <row r="499" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A499" s="1">
+        <v>46105</v>
+      </c>
+      <c r="C499">
+        <v>4610.8718719999997</v>
+      </c>
+      <c r="D499">
+        <v>4633.1175869999997</v>
+      </c>
+      <c r="E499">
+        <v>4471.4768270000004</v>
+      </c>
+      <c r="F499">
+        <v>4502.5689000000002</v>
+      </c>
+      <c r="G499">
+        <v>4349.3154889999996</v>
+      </c>
+      <c r="H499">
+        <v>4254.3052360000001</v>
+      </c>
+      <c r="I499">
+        <v>4291.7446170000003</v>
+      </c>
+      <c r="J499">
+        <v>4263.3648709999998</v>
+      </c>
+      <c r="K499">
+        <v>4128.9725619999999</v>
+      </c>
+      <c r="L499">
+        <v>4143.3177560000004</v>
+      </c>
+      <c r="M499">
+        <v>4030.6657890000001</v>
+      </c>
+      <c r="N499">
+        <v>4071.6381489999999</v>
+      </c>
+      <c r="O499">
+        <v>3964.243923</v>
+      </c>
+    </row>
+    <row r="500" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A500" s="1">
+        <v>46106</v>
+      </c>
+      <c r="C500">
+        <v>4612.2808420000001</v>
+      </c>
+      <c r="D500">
+        <v>4636.7648209999998</v>
+      </c>
+      <c r="E500">
+        <v>4477.1923420000003</v>
+      </c>
+      <c r="F500">
+        <v>4508.3862300000001</v>
+      </c>
+      <c r="G500">
+        <v>4356.0662030000003</v>
+      </c>
+      <c r="H500">
+        <v>4265.4940290000004</v>
+      </c>
+      <c r="I500">
+        <v>4302.8877419999999</v>
+      </c>
+      <c r="J500">
+        <v>4270.9009070000002</v>
+      </c>
+      <c r="K500">
+        <v>4131.4952519999997</v>
+      </c>
+      <c r="L500">
+        <v>4152.4364729999998</v>
+      </c>
+      <c r="M500">
+        <v>4037.1809239999998</v>
+      </c>
+      <c r="N500">
+        <v>4069.9189719999999</v>
+      </c>
+      <c r="O500">
+        <v>3968.1527970000002</v>
+      </c>
+    </row>
+    <row r="501" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A501" s="1">
+        <v>46107</v>
+      </c>
+      <c r="C501">
+        <v>4621.8108700000003</v>
+      </c>
+      <c r="D501">
+        <v>4637.4401850000004</v>
+      </c>
+      <c r="E501">
+        <v>4470.5126140000002</v>
+      </c>
+      <c r="F501">
+        <v>4501.3770320000003</v>
+      </c>
+      <c r="G501">
+        <v>4347.1198729999996</v>
+      </c>
+      <c r="H501">
+        <v>4251.0622000000003</v>
+      </c>
+      <c r="I501">
+        <v>4287.8722500000003</v>
+      </c>
+      <c r="J501">
+        <v>4256.2379609999998</v>
+      </c>
+      <c r="K501">
+        <v>4113.1995889999998</v>
+      </c>
+      <c r="L501">
+        <v>4129.914143</v>
+      </c>
+      <c r="M501">
+        <v>4015.282166</v>
+      </c>
+      <c r="N501">
+        <v>4046.6706530000001</v>
+      </c>
+      <c r="O501">
+        <v>3945.2841720000001</v>
+      </c>
+    </row>
+    <row r="502" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A502" s="1">
+        <v>46108</v>
+      </c>
+      <c r="C502">
+        <v>4627.1853959999999</v>
+      </c>
+      <c r="D502">
+        <v>4643.8525950000003</v>
+      </c>
+      <c r="E502">
+        <v>4478.3654720000004</v>
+      </c>
+      <c r="F502">
+        <v>4509.6507389999997</v>
+      </c>
+      <c r="G502">
+        <v>4354.6369549999999</v>
+      </c>
+      <c r="H502">
+        <v>4256.9152169999998</v>
+      </c>
+      <c r="I502">
+        <v>4292.7494640000004</v>
+      </c>
+      <c r="J502">
+        <v>4266.9053139999996</v>
+      </c>
+      <c r="K502">
+        <v>4129.683196</v>
+      </c>
+      <c r="L502">
+        <v>4141.6852520000002</v>
+      </c>
+      <c r="M502">
+        <v>4023.5047239999999</v>
+      </c>
+      <c r="N502">
+        <v>4054.5530180000001</v>
+      </c>
+      <c r="O502">
+        <v>3952.9699909999999</v>
+      </c>
+    </row>
+    <row r="503" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A503" s="1">
+        <v>46111</v>
+      </c>
+      <c r="C503">
+        <v>4632.3793919999998</v>
+      </c>
+      <c r="D503">
+        <v>4656.7727400000003</v>
+      </c>
+      <c r="E503">
+        <v>4492.8659930000003</v>
+      </c>
+      <c r="F503">
+        <v>4522.3350899999996</v>
+      </c>
+      <c r="G503">
+        <v>4368.8308420000003</v>
+      </c>
+      <c r="H503">
+        <v>4271.1970270000002</v>
+      </c>
+      <c r="I503">
+        <v>4308.3122860000003</v>
+      </c>
+      <c r="J503">
+        <v>4273.7767350000004</v>
+      </c>
+      <c r="K503">
+        <v>4125.3389399999996</v>
+      </c>
+      <c r="L503">
+        <v>4141.1704460000001</v>
+      </c>
+      <c r="M503">
+        <v>4028.3651589999999</v>
+      </c>
+      <c r="N503">
+        <v>4057.2950740000001</v>
+      </c>
+      <c r="O503">
+        <v>3961.7389699999999</v>
+      </c>
+    </row>
+    <row r="504" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A504" s="1">
+        <v>46112</v>
+      </c>
+      <c r="C504">
+        <v>4635.288716</v>
+      </c>
+      <c r="D504">
+        <v>4665.386152</v>
+      </c>
+      <c r="E504">
+        <v>4511.262917</v>
+      </c>
+      <c r="F504">
+        <v>4542.7087629999996</v>
+      </c>
+      <c r="G504">
+        <v>4396.699235</v>
+      </c>
+      <c r="H504">
+        <v>4305.5234870000004</v>
+      </c>
+      <c r="I504">
+        <v>4343.7857759999997</v>
+      </c>
+      <c r="J504">
+        <v>4307.8204329999999</v>
+      </c>
+      <c r="K504">
+        <v>4145.1650200000004</v>
+      </c>
+      <c r="L504">
+        <v>4172.6400309999999</v>
+      </c>
+      <c r="M504">
+        <v>4061.4938699999998</v>
+      </c>
+      <c r="N504">
+        <v>4093.878952</v>
+      </c>
+      <c r="O504">
+        <v>4002.7590009999999</v>
+      </c>
+    </row>
+    <row r="505" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A505" s="1">
+        <v>46113</v>
+      </c>
+      <c r="C505">
+        <v>4640.2413759999999</v>
+      </c>
+      <c r="D505">
+        <v>4671.0094319999998</v>
+      </c>
+      <c r="E505">
+        <v>4518.5459259999998</v>
+      </c>
+      <c r="F505">
+        <v>4549.6628259999998</v>
+      </c>
+      <c r="G505">
+        <v>4403.9901529999997</v>
+      </c>
+      <c r="H505">
+        <v>4315.4442010000002</v>
+      </c>
+      <c r="I505">
+        <v>4354.2263700000003</v>
+      </c>
+      <c r="J505">
+        <v>4316.1465410000001</v>
+      </c>
+      <c r="K505">
+        <v>4156.9573200000004</v>
+      </c>
+      <c r="L505">
+        <v>4182.8369060000005</v>
+      </c>
+      <c r="M505">
+        <v>4078.5929660000002</v>
+      </c>
+      <c r="N505">
+        <v>4116.7239589999999</v>
+      </c>
+      <c r="O505">
+        <v>4020.5359939999998</v>
+      </c>
+    </row>
+    <row r="506" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A506" s="1">
+        <v>46114</v>
+      </c>
+      <c r="C506">
+        <v>4646.7136680000003</v>
+      </c>
+      <c r="D506">
+        <v>4676.28701</v>
+      </c>
+      <c r="E506">
+        <v>4520.6640450000004</v>
+      </c>
+      <c r="F506">
+        <v>4549.8465500000002</v>
+      </c>
+      <c r="G506">
+        <v>4400.6165629999996</v>
+      </c>
+      <c r="H506">
+        <v>4309.7469330000004</v>
+      </c>
+      <c r="I506">
+        <v>4348.709672</v>
+      </c>
+      <c r="J506">
+        <v>4311.6592440000004</v>
+      </c>
+      <c r="K506">
+        <v>4154.9335600000004</v>
+      </c>
+      <c r="L506">
+        <v>4193.1006649999999</v>
+      </c>
+      <c r="M506">
+        <v>4081.0467330000001</v>
+      </c>
+      <c r="N506">
+        <v>4120.9121189999996</v>
+      </c>
+      <c r="O506">
+        <v>4027.930108</v>
+      </c>
+    </row>
+    <row r="507" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A507" s="1">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="508" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A508" s="1">
+        <v>46118</v>
+      </c>
+      <c r="C508">
+        <v>4648.4981690000004</v>
+      </c>
+      <c r="D508">
+        <v>4676.6758499999996</v>
+      </c>
+      <c r="E508">
+        <v>4518.0542169999999</v>
+      </c>
+      <c r="F508">
+        <v>4547.9447140000002</v>
+      </c>
+      <c r="G508">
+        <v>4400.2748620000002</v>
+      </c>
+      <c r="H508">
+        <v>4311.906602</v>
+      </c>
+      <c r="I508">
+        <v>4352.1019189999997</v>
+      </c>
+      <c r="J508">
+        <v>4312.9631490000002</v>
+      </c>
+      <c r="K508">
+        <v>4159.079686</v>
+      </c>
+      <c r="L508">
+        <v>4204.4925750000002</v>
+      </c>
+      <c r="M508">
+        <v>4100.3040410000003</v>
+      </c>
+      <c r="N508">
+        <v>4144.9536099999996</v>
+      </c>
+      <c r="O508">
+        <v>4045.8104349999999</v>
+      </c>
+    </row>
+    <row r="509" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A509" s="1">
+        <v>46119</v>
+      </c>
+      <c r="C509">
+        <v>4652.7603159999999</v>
+      </c>
+      <c r="D509">
+        <v>4679.3598089999996</v>
+      </c>
+      <c r="E509">
+        <v>4518.9527109999999</v>
+      </c>
+      <c r="F509">
+        <v>4546.9629599999998</v>
+      </c>
+      <c r="G509">
+        <v>4396.1378260000001</v>
+      </c>
+      <c r="H509">
+        <v>4310.1096719999996</v>
+      </c>
+      <c r="I509">
+        <v>4349.2336949999999</v>
+      </c>
+      <c r="J509">
+        <v>4308.9037790000002</v>
+      </c>
+      <c r="K509">
+        <v>4162.8975620000001</v>
+      </c>
+      <c r="L509">
+        <v>4204.4426830000002</v>
+      </c>
+      <c r="M509">
+        <v>4099.6789509999999</v>
+      </c>
+      <c r="N509">
+        <v>4142.5417090000001</v>
+      </c>
+      <c r="O509">
+        <v>4046.1307670000001</v>
+      </c>
+    </row>
+    <row r="510" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A510" s="1">
+        <v>46120</v>
+      </c>
+      <c r="C510">
+        <v>4651.8828960000001</v>
+      </c>
+      <c r="D510">
+        <v>4683.0836749999999</v>
+      </c>
+      <c r="E510">
+        <v>4534.1918249999999</v>
+      </c>
+      <c r="F510">
+        <v>4568.2756140000001</v>
+      </c>
+      <c r="G510">
+        <v>4427.8138900000004</v>
+      </c>
+      <c r="H510">
+        <v>4341.8825020000004</v>
+      </c>
+      <c r="I510">
+        <v>4382.9991570000002</v>
+      </c>
+      <c r="J510">
+        <v>4341.2770229999996</v>
+      </c>
+      <c r="K510">
+        <v>4196.996126</v>
+      </c>
+      <c r="L510">
+        <v>4238.1733299999996</v>
+      </c>
+      <c r="M510">
+        <v>4135.386348</v>
+      </c>
+      <c r="N510">
+        <v>4178.9342329999999</v>
+      </c>
+      <c r="O510">
+        <v>4087.423127</v>
+      </c>
+    </row>
+    <row r="511" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A511" s="1">
+        <v>46121</v>
+      </c>
+      <c r="C511">
+        <v>4656.4601579999999</v>
+      </c>
+      <c r="D511">
+        <v>4686.9539500000001</v>
+      </c>
+      <c r="E511">
+        <v>4541.1242069999998</v>
+      </c>
+      <c r="F511">
+        <v>4576.9014150000003</v>
+      </c>
+      <c r="G511">
+        <v>4433.2940609999996</v>
+      </c>
+      <c r="H511">
+        <v>4346.0338300000003</v>
+      </c>
+      <c r="I511">
+        <v>4388.6785460000001</v>
+      </c>
+      <c r="J511">
+        <v>4349.4536070000004</v>
+      </c>
+      <c r="K511">
+        <v>4208.0453479999996</v>
+      </c>
+      <c r="L511">
+        <v>4248.0716519999996</v>
+      </c>
+      <c r="M511">
+        <v>4146.7828790000003</v>
+      </c>
+      <c r="N511">
+        <v>4193.8257830000002</v>
+      </c>
+      <c r="O511">
+        <v>4104.5295260000003</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -44901,7 +46049,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE81DAD-ED15-4633-A0F7-1D8C32328F6D}">
-  <dimension ref="A1:Z497"/>
+  <dimension ref="A1:Z511"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -66877,6 +68025,583 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
+    <row r="498" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A498" s="1">
+        <v>46104</v>
+      </c>
+      <c r="D498">
+        <v>-2.6800000000000001E-2</v>
+      </c>
+      <c r="E498">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="F498">
+        <v>9.5999999999999992E-3</v>
+      </c>
+      <c r="G498">
+        <v>1.44E-2</v>
+      </c>
+      <c r="H498">
+        <v>2.46E-2</v>
+      </c>
+      <c r="I498">
+        <v>4.1300000000000003E-2</v>
+      </c>
+      <c r="J498">
+        <v>5.3600000000000002E-2</v>
+      </c>
+      <c r="K498">
+        <v>7.1499999999999994E-2</v>
+      </c>
+      <c r="L498">
+        <v>7.5700000000000003E-2</v>
+      </c>
+      <c r="M498">
+        <v>8.3500000000000005E-2</v>
+      </c>
+      <c r="N498">
+        <v>8.3799999999999999E-2</v>
+      </c>
+      <c r="O498">
+        <v>9.35E-2</v>
+      </c>
+      <c r="P498">
+        <v>9.6600000000000005E-2</v>
+      </c>
+    </row>
+    <row r="499" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A499" s="1">
+        <v>46105</v>
+      </c>
+      <c r="D499">
+        <v>-2.7E-2</v>
+      </c>
+      <c r="E499">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="F499">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="G499">
+        <v>1.44E-2</v>
+      </c>
+      <c r="H499">
+        <v>2.47E-2</v>
+      </c>
+      <c r="I499">
+        <v>4.1099999999999998E-2</v>
+      </c>
+      <c r="J499">
+        <v>5.3900000000000003E-2</v>
+      </c>
+      <c r="K499">
+        <v>7.0300000000000001E-2</v>
+      </c>
+      <c r="L499">
+        <v>7.4899999999999994E-2</v>
+      </c>
+      <c r="M499">
+        <v>8.2900000000000001E-2</v>
+      </c>
+      <c r="N499">
+        <v>8.3400000000000002E-2</v>
+      </c>
+      <c r="O499">
+        <v>9.3200000000000005E-2</v>
+      </c>
+      <c r="P499">
+        <v>9.64E-2</v>
+      </c>
+    </row>
+    <row r="500" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A500" s="1">
+        <v>46106</v>
+      </c>
+      <c r="D500">
+        <v>-3.4599999999999999E-2</v>
+      </c>
+      <c r="E500">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="F500">
+        <v>8.6999999999999994E-3</v>
+      </c>
+      <c r="G500">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="H500">
+        <v>2.4500000000000001E-2</v>
+      </c>
+      <c r="I500">
+        <v>4.0500000000000001E-2</v>
+      </c>
+      <c r="J500">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="K500">
+        <v>6.7500000000000004E-2</v>
+      </c>
+      <c r="L500">
+        <v>7.0699999999999999E-2</v>
+      </c>
+      <c r="M500">
+        <v>8.0299999999999996E-2</v>
+      </c>
+      <c r="N500">
+        <v>8.2100000000000006E-2</v>
+      </c>
+      <c r="O500">
+        <v>9.2600000000000002E-2</v>
+      </c>
+      <c r="P500">
+        <v>9.5799999999999996E-2</v>
+      </c>
+    </row>
+    <row r="501" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A501" s="1">
+        <v>46107</v>
+      </c>
+      <c r="D501">
+        <v>-5.0999999999999997E-2</v>
+      </c>
+      <c r="E501">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="F501">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="G501">
+        <v>1.43E-2</v>
+      </c>
+      <c r="H501">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="I501">
+        <v>4.02E-2</v>
+      </c>
+      <c r="J501">
+        <v>5.2400000000000002E-2</v>
+      </c>
+      <c r="K501">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="L501">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="M501">
+        <v>7.7299999999999994E-2</v>
+      </c>
+      <c r="N501">
+        <v>7.9399999999999998E-2</v>
+      </c>
+      <c r="O501">
+        <v>9.0899999999999995E-2</v>
+      </c>
+      <c r="P501">
+        <v>9.4799999999999995E-2</v>
+      </c>
+    </row>
+    <row r="502" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A502" s="1">
+        <v>46108</v>
+      </c>
+      <c r="D502">
+        <v>-5.0099999999999999E-2</v>
+      </c>
+      <c r="E502">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="F502">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="G502">
+        <v>1.43E-2</v>
+      </c>
+      <c r="H502">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="I502">
+        <v>0.04</v>
+      </c>
+      <c r="J502">
+        <v>5.2600000000000001E-2</v>
+      </c>
+      <c r="K502">
+        <v>6.4500000000000002E-2</v>
+      </c>
+      <c r="L502">
+        <v>6.8000000000000005E-2</v>
+      </c>
+      <c r="M502">
+        <v>7.5899999999999995E-2</v>
+      </c>
+      <c r="N502">
+        <v>7.9100000000000004E-2</v>
+      </c>
+      <c r="O502">
+        <v>9.0499999999999997E-2</v>
+      </c>
+      <c r="P502">
+        <v>9.4399999999999998E-2</v>
+      </c>
+    </row>
+    <row r="503" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A503" s="1">
+        <v>46111</v>
+      </c>
+      <c r="D503">
+        <v>-4.9299999999999997E-2</v>
+      </c>
+      <c r="E503">
+        <v>0</v>
+      </c>
+      <c r="F503">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="G503">
+        <v>1.44E-2</v>
+      </c>
+      <c r="H503">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="I503">
+        <v>0.04</v>
+      </c>
+      <c r="J503">
+        <v>5.2400000000000002E-2</v>
+      </c>
+      <c r="K503">
+        <v>6.4299999999999996E-2</v>
+      </c>
+      <c r="L503">
+        <v>6.7799999999999999E-2</v>
+      </c>
+      <c r="M503">
+        <v>7.4300000000000005E-2</v>
+      </c>
+      <c r="N503">
+        <v>7.6100000000000001E-2</v>
+      </c>
+      <c r="O503">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="P503">
+        <v>9.3700000000000006E-2</v>
+      </c>
+    </row>
+    <row r="504" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A504" s="1">
+        <v>46112</v>
+      </c>
+      <c r="D504">
+        <v>-4.2299999999999997E-2</v>
+      </c>
+      <c r="E504">
+        <v>-2.7000000000000001E-3</v>
+      </c>
+      <c r="F504">
+        <v>7.4999999999999997E-3</v>
+      </c>
+      <c r="G504">
+        <v>1.44E-2</v>
+      </c>
+      <c r="H504">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="I504">
+        <v>0.04</v>
+      </c>
+      <c r="J504">
+        <v>5.3100000000000001E-2</v>
+      </c>
+      <c r="K504">
+        <v>6.4299999999999996E-2</v>
+      </c>
+      <c r="L504">
+        <v>6.7799999999999999E-2</v>
+      </c>
+      <c r="M504">
+        <v>7.4200000000000002E-2</v>
+      </c>
+      <c r="N504">
+        <v>7.4800000000000005E-2</v>
+      </c>
+      <c r="O504">
+        <v>8.8499999999999995E-2</v>
+      </c>
+      <c r="P504">
+        <v>9.3399999999999997E-2</v>
+      </c>
+    </row>
+    <row r="505" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A505" s="1">
+        <v>46113</v>
+      </c>
+      <c r="D505">
+        <v>-3.3500000000000002E-2</v>
+      </c>
+      <c r="E505">
+        <v>-3.0000000000000001E-3</v>
+      </c>
+      <c r="F505">
+        <v>6.6E-3</v>
+      </c>
+      <c r="G505">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="H505">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="I505">
+        <v>0.04</v>
+      </c>
+      <c r="J505">
+        <v>5.3100000000000001E-2</v>
+      </c>
+      <c r="K505">
+        <v>6.4100000000000004E-2</v>
+      </c>
+      <c r="L505">
+        <v>6.7599999999999993E-2</v>
+      </c>
+      <c r="M505">
+        <v>7.4099999999999999E-2</v>
+      </c>
+      <c r="N505">
+        <v>7.46E-2</v>
+      </c>
+      <c r="O505">
+        <v>8.72E-2</v>
+      </c>
+      <c r="P505">
+        <v>9.3299999999999994E-2</v>
+      </c>
+    </row>
+    <row r="506" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A506" s="1">
+        <v>46114</v>
+      </c>
+      <c r="D506">
+        <v>-2.5899999999999999E-2</v>
+      </c>
+      <c r="E506">
+        <v>-2.8E-3</v>
+      </c>
+      <c r="F506">
+        <v>6.4999999999999997E-3</v>
+      </c>
+      <c r="G506">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="H506">
+        <v>2.5499999999999998E-2</v>
+      </c>
+      <c r="I506">
+        <v>0.04</v>
+      </c>
+      <c r="J506">
+        <v>5.2499999999999998E-2</v>
+      </c>
+      <c r="K506">
+        <v>6.4199999999999993E-2</v>
+      </c>
+      <c r="L506">
+        <v>6.7400000000000002E-2</v>
+      </c>
+      <c r="M506">
+        <v>7.3499999999999996E-2</v>
+      </c>
+      <c r="N506">
+        <v>7.4099999999999999E-2</v>
+      </c>
+      <c r="O506">
+        <v>8.6699999999999999E-2</v>
+      </c>
+      <c r="P506">
+        <v>9.3200000000000005E-2</v>
+      </c>
+    </row>
+    <row r="507" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A507" s="1">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="508" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A508" s="1">
+        <v>46118</v>
+      </c>
+      <c r="D508">
+        <v>-2.1000000000000001E-2</v>
+      </c>
+      <c r="E508">
+        <v>-1.2999999999999999E-3</v>
+      </c>
+      <c r="F508">
+        <v>6.4999999999999997E-3</v>
+      </c>
+      <c r="G508">
+        <v>1.4800000000000001E-2</v>
+      </c>
+      <c r="H508">
+        <v>2.5499999999999998E-2</v>
+      </c>
+      <c r="I508">
+        <v>0.04</v>
+      </c>
+      <c r="J508">
+        <v>5.2499999999999998E-2</v>
+      </c>
+      <c r="K508">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="L508">
+        <v>6.7400000000000002E-2</v>
+      </c>
+      <c r="M508">
+        <v>7.3499999999999996E-2</v>
+      </c>
+      <c r="N508">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="O508">
+        <v>8.6199999999999999E-2</v>
+      </c>
+      <c r="P508">
+        <v>9.2899999999999996E-2</v>
+      </c>
+    </row>
+    <row r="509" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A509" s="1">
+        <v>46119</v>
+      </c>
+      <c r="D509">
+        <v>-1.7600000000000001E-2</v>
+      </c>
+      <c r="E509">
+        <v>0</v>
+      </c>
+      <c r="F509">
+        <v>6.6E-3</v>
+      </c>
+      <c r="G509">
+        <v>1.44E-2</v>
+      </c>
+      <c r="H509">
+        <v>2.52E-2</v>
+      </c>
+      <c r="I509">
+        <v>3.9899999999999998E-2</v>
+      </c>
+      <c r="J509">
+        <v>5.2499999999999998E-2</v>
+      </c>
+      <c r="K509">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="L509">
+        <v>6.7400000000000002E-2</v>
+      </c>
+      <c r="M509">
+        <v>7.3499999999999996E-2</v>
+      </c>
+      <c r="N509">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="O509">
+        <v>8.6099999999999996E-2</v>
+      </c>
+      <c r="P509">
+        <v>9.2899999999999996E-2</v>
+      </c>
+    </row>
+    <row r="510" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A510" s="1">
+        <v>46120</v>
+      </c>
+      <c r="D510">
+        <v>-1.2999999999999999E-2</v>
+      </c>
+      <c r="E510">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="F510">
+        <v>8.6E-3</v>
+      </c>
+      <c r="G510">
+        <v>1.44E-2</v>
+      </c>
+      <c r="H510">
+        <v>2.53E-2</v>
+      </c>
+      <c r="I510">
+        <v>4.0099999999999997E-2</v>
+      </c>
+      <c r="J510">
+        <v>5.2499999999999998E-2</v>
+      </c>
+      <c r="K510">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="L510">
+        <v>6.7500000000000004E-2</v>
+      </c>
+      <c r="M510">
+        <v>7.3499999999999996E-2</v>
+      </c>
+      <c r="N510">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="O510">
+        <v>8.5999999999999993E-2</v>
+      </c>
+      <c r="P510">
+        <v>9.2899999999999996E-2</v>
+      </c>
+    </row>
+    <row r="511" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A511" s="1">
+        <v>46121</v>
+      </c>
+      <c r="D511">
+        <v>-1.01E-2</v>
+      </c>
+      <c r="E511">
+        <v>3.3E-3</v>
+      </c>
+      <c r="F511">
+        <v>8.8000000000000005E-3</v>
+      </c>
+      <c r="G511">
+        <v>1.44E-2</v>
+      </c>
+      <c r="H511">
+        <v>2.53E-2</v>
+      </c>
+      <c r="I511">
+        <v>4.0500000000000001E-2</v>
+      </c>
+      <c r="J511">
+        <v>5.2699999999999997E-2</v>
+      </c>
+      <c r="K511">
+        <v>6.4100000000000004E-2</v>
+      </c>
+      <c r="L511">
+        <v>6.7500000000000004E-2</v>
+      </c>
+      <c r="M511">
+        <v>7.3499999999999996E-2</v>
+      </c>
+      <c r="N511">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="O511">
+        <v>8.5999999999999993E-2</v>
+      </c>
+      <c r="P511">
+        <v>9.2999999999999999E-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Dash Hedge IPCA - 2026-04-23
</commit_message>
<xml_diff>
--- a/Dados/Atualizar.xlsx
+++ b/Dados/Atualizar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\livia.jacob\Desktop\Hedge IPCA teste\Projeto-Hedge-IPCA\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D624B7C6-5BF2-491A-B22C-A16FDCC4AE13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F5757B-DE1B-4421-8E3D-740B8559EB70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-1260" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -18,52 +18,52 @@
     <sheet name="Planilha2" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_ECO_RANGE_ID00e76574b0624b3f80d0e29bd2420585" localSheetId="2" hidden="1">Planilha2!$I$4:$I$511</definedName>
-    <definedName name="_ECO_RANGE_ID0ca2184d708a4271baf003d9a1c716da" localSheetId="1" hidden="1">Planilha1!$B$3</definedName>
-    <definedName name="_ECO_RANGE_ID1c21957cb5054573a1d238750a58a67e" localSheetId="1" hidden="1">Planilha1!$A$4:$B$511</definedName>
-    <definedName name="_ECO_RANGE_ID1d28d9a8f21f494e8ce2ea4d34ae2699" localSheetId="1" hidden="1">Planilha1!$K$4:$K$511</definedName>
-    <definedName name="_ECO_RANGE_ID1e171e8255724b69b1039f752a0c6357" localSheetId="2" hidden="1">Planilha2!$P$4:$P$511</definedName>
-    <definedName name="_ECO_RANGE_ID1f847766b5984ccf829f829bbee3c277" localSheetId="2" hidden="1">Planilha2!$J$4:$J$511</definedName>
-    <definedName name="_ECO_RANGE_ID2263af481ec0463180d115747aa43df9" localSheetId="1" hidden="1">Planilha1!$J$4:$J$511</definedName>
-    <definedName name="_ECO_RANGE_ID232ebef712f94d0b81b56c536489891c" localSheetId="0" hidden="1">Plan1!$F$4:$F$511</definedName>
-    <definedName name="_ECO_RANGE_ID2456f6dbaf9a46f9a7a8da48def4aaa5" localSheetId="0" hidden="1">Plan1!$G$4:$G$511</definedName>
-    <definedName name="_ECO_RANGE_ID254e87af413c4cb986cdc16f2c5dffae" localSheetId="2" hidden="1">Planilha2!$O$4:$O$511</definedName>
-    <definedName name="_ECO_RANGE_ID2857e1655bd94ecda14895a570f07374" localSheetId="2" hidden="1">Planilha2!$M$4:$M$511</definedName>
-    <definedName name="_ECO_RANGE_ID2bf3f203bdd04613a6363ea76bf46229" localSheetId="2" hidden="1">Planilha2!$C$4:$C$511</definedName>
-    <definedName name="_ECO_RANGE_ID3937a644b00e41c18364273ec40793bc" localSheetId="0" hidden="1">Plan1!$L$4:$L$511</definedName>
-    <definedName name="_ECO_RANGE_ID3b23869efc324a4abe9ccfbb4b298e60" localSheetId="1" hidden="1">Planilha1!$L$4:$L$511</definedName>
-    <definedName name="_ECO_RANGE_ID3b743473a33142c6b9458acec2a37261" localSheetId="1" hidden="1">Planilha1!$E$4:$E$511</definedName>
-    <definedName name="_ECO_RANGE_ID473fe07ab4704df8bffef6945131b806" localSheetId="0" hidden="1">Plan1!$J$4:$J$511</definedName>
-    <definedName name="_ECO_RANGE_ID47b5330b869b40ebb1412c1f212c5686" localSheetId="0" hidden="1">Plan1!$I$4:$I$511</definedName>
-    <definedName name="_ECO_RANGE_ID54af0d7ac46f4f83a05fbe311eb66f59" localSheetId="0" hidden="1">Plan1!$E$4:$E$511</definedName>
-    <definedName name="_ECO_RANGE_ID5b747179ed9b40c090504187252e6c12" localSheetId="2" hidden="1">Planilha2!$N$4:$N$511</definedName>
-    <definedName name="_ECO_RANGE_ID5e9abdc0d24d42d582f711ff881e0cc7" localSheetId="2" hidden="1">Planilha2!$H$4:$H$511</definedName>
-    <definedName name="_ECO_RANGE_ID6b39f817d71a492b8d4a3485ec2533e8" localSheetId="0" hidden="1">Plan1!$C$4:$C$511</definedName>
-    <definedName name="_ECO_RANGE_ID6d5830ca54f24720bb7fa7ab018c5b91" localSheetId="2" hidden="1">Planilha2!$B$3</definedName>
-    <definedName name="_ECO_RANGE_ID77ac73d043e24720b080ca54f777d98d" localSheetId="1" hidden="1">Planilha1!$F$4:$F$511</definedName>
-    <definedName name="_ECO_RANGE_ID7cfb044391844e06ba8843b0d19da22f" localSheetId="2" hidden="1">Planilha2!$K$4:$K$511</definedName>
-    <definedName name="_ECO_RANGE_ID7d562063ae1843d699e06abbad50c403" localSheetId="0" hidden="1">Plan1!$K$4:$K$511</definedName>
-    <definedName name="_ECO_RANGE_ID7d8b621180af48ebbbc3c410be289395" localSheetId="1" hidden="1">Planilha1!$D$4:$D$511</definedName>
-    <definedName name="_ECO_RANGE_ID7daf296a8e4c4c26a5d2bde7a75c235e" localSheetId="0" hidden="1">Plan1!$M$4:$M$511</definedName>
-    <definedName name="_ECO_RANGE_ID9aabd0f32504463a96b4226636091fb2" localSheetId="2" hidden="1">Planilha2!$A$4:$B$511</definedName>
-    <definedName name="_ECO_RANGE_ID9d45bf1d2cab443db565260ba3806640" localSheetId="0" hidden="1">Plan1!$D$4:$D$511</definedName>
-    <definedName name="_ECO_RANGE_ID9ecd5d7c51554ce6ba1480d8c3eee854" localSheetId="2" hidden="1">Planilha2!$E$4:$E$511</definedName>
-    <definedName name="_ECO_RANGE_IDa12df9e429f44a729e21711af60e42e8" localSheetId="0" hidden="1">Plan1!$N$4:$N$511</definedName>
-    <definedName name="_ECO_RANGE_IDa887542f3b7846f2afb9502f13811566" localSheetId="0" hidden="1">Plan1!$O$4:$O$511</definedName>
-    <definedName name="_ECO_RANGE_IDab70849247ca481896605025d66a800b" localSheetId="1" hidden="1">Planilha1!$N$4:$N$511</definedName>
-    <definedName name="_ECO_RANGE_IDad723ae37f574a4197d1df789db1c529" localSheetId="1" hidden="1">Planilha1!$O$4:$O$511</definedName>
-    <definedName name="_ECO_RANGE_IDb804cfc80e9043d9af304e043a31d260" localSheetId="0" hidden="1">Plan1!$B$3</definedName>
-    <definedName name="_ECO_RANGE_IDb96a28ff555545e4aaaebc6c701a168d" localSheetId="2" hidden="1">Planilha2!$F$4:$F$511</definedName>
-    <definedName name="_ECO_RANGE_IDc7b478ef50304093bb8e5bf40a17c94c" localSheetId="2" hidden="1">Planilha2!$G$4:$G$511</definedName>
-    <definedName name="_ECO_RANGE_IDcdd812b56b634f0e819953c5e571c66e" localSheetId="1" hidden="1">Planilha1!$I$4:$I$511</definedName>
-    <definedName name="_ECO_RANGE_IDd061a8b7d8714484b222e53980f0e91a" localSheetId="1" hidden="1">Planilha1!$H$4:$H$511</definedName>
-    <definedName name="_ECO_RANGE_IDd5577f4583464d118628ec8007f31230" localSheetId="1" hidden="1">Planilha1!$G$4:$G$511</definedName>
-    <definedName name="_ECO_RANGE_IDda57c28fb56c4536913e96798d0e8fb6" localSheetId="0" hidden="1">Plan1!$H$4:$H$511</definedName>
-    <definedName name="_ECO_RANGE_IDe31d00163de0498c9ac7cb0a33c5a73f" localSheetId="0" hidden="1">Plan1!$A$4:$B$511</definedName>
-    <definedName name="_ECO_RANGE_IDe3fe4b7a712d41c48173b5ff41e2769e" localSheetId="1" hidden="1">Planilha1!$C$4:$C$511</definedName>
-    <definedName name="_ECO_RANGE_IDe9544339a6694282ab37faa936de2ab2" localSheetId="2" hidden="1">Planilha2!$L$4:$L$511</definedName>
-    <definedName name="_ECO_RANGE_IDf58054575add4fd2a046a2c25a6473e7" localSheetId="2" hidden="1">Planilha2!$D$4:$D$511</definedName>
-    <definedName name="_ECO_RANGE_IDf7a9036fd4df40249838f740cd819492" localSheetId="1" hidden="1">Planilha1!$M$4:$M$511</definedName>
+    <definedName name="_ECO_RANGE_ID010b73370d3d4594bd56d1130fb44ae1" localSheetId="2" hidden="1">Planilha2!$M$4:$M$520</definedName>
+    <definedName name="_ECO_RANGE_ID028d92a724a1460397fcd1fa2784194e" localSheetId="1" hidden="1">Planilha1!$D$4:$D$520</definedName>
+    <definedName name="_ECO_RANGE_ID0961c7db7f564b5f82c625929c18801a" localSheetId="0" hidden="1">Plan1!$I$4:$I$520</definedName>
+    <definedName name="_ECO_RANGE_ID116df8a3fe974e4cbfab46b7737c3964" localSheetId="0" hidden="1">Plan1!$A$4:$B$520</definedName>
+    <definedName name="_ECO_RANGE_ID11eccfa2166b48c7a796d6e24b29b4ae" localSheetId="1" hidden="1">Planilha1!$N$4:$N$520</definedName>
+    <definedName name="_ECO_RANGE_ID15af4835f4b3476389b11cef426f7bfd" localSheetId="2" hidden="1">Planilha2!$I$4:$I$520</definedName>
+    <definedName name="_ECO_RANGE_ID18829721627b4d9c90db96de34b06591" localSheetId="1" hidden="1">Planilha1!$J$4:$J$520</definedName>
+    <definedName name="_ECO_RANGE_ID2b203464bab34ecb975e08be97d6475e" localSheetId="2" hidden="1">Planilha2!$N$4:$N$520</definedName>
+    <definedName name="_ECO_RANGE_ID398d4eb9c72440578edfc4724dd06f12" localSheetId="2" hidden="1">Planilha2!$F$4:$F$520</definedName>
+    <definedName name="_ECO_RANGE_ID407b129d06af4587aebdc2330b41cc3e" localSheetId="0" hidden="1">Plan1!$E$4:$E$520</definedName>
+    <definedName name="_ECO_RANGE_ID4aadcd8461084af0bf87ddbdadd85757" localSheetId="0" hidden="1">Plan1!$J$4:$J$520</definedName>
+    <definedName name="_ECO_RANGE_ID4f4cd9cd38d244749ca0f56c4145f501" localSheetId="2" hidden="1">Planilha2!$L$4:$L$520</definedName>
+    <definedName name="_ECO_RANGE_ID540461f8ac8a4b989069f6c5bc5e9319" localSheetId="0" hidden="1">Plan1!$G$4:$G$520</definedName>
+    <definedName name="_ECO_RANGE_ID580b88c1f9344e7b85e2e69f8bcb385b" localSheetId="1" hidden="1">Planilha1!$K$4:$K$520</definedName>
+    <definedName name="_ECO_RANGE_ID5cd3bf4d86234c488d8b1bb5fd382906" localSheetId="2" hidden="1">Planilha2!$H$4:$H$520</definedName>
+    <definedName name="_ECO_RANGE_ID5ea3e058554c4a1cbb098f2978d3bff4" localSheetId="0" hidden="1">Plan1!$C$4:$C$520</definedName>
+    <definedName name="_ECO_RANGE_ID612846aa44134091abb67e8d977bef80" localSheetId="1" hidden="1">Planilha1!$O$4:$O$520</definedName>
+    <definedName name="_ECO_RANGE_ID6d92d3f8a4384ebaa9196bbdd2a0dbd9" localSheetId="1" hidden="1">Planilha1!$C$4:$C$520</definedName>
+    <definedName name="_ECO_RANGE_ID6f1ed0eec9b346cbbfb023171a8a9584" localSheetId="2" hidden="1">Planilha2!$B$3</definedName>
+    <definedName name="_ECO_RANGE_ID75ef71a5f31742d9b5c7e8f4114a2bf4" localSheetId="2" hidden="1">Planilha2!$A$4:$B$520</definedName>
+    <definedName name="_ECO_RANGE_ID76f6a5ac1208437aad49a2c2ebda6e44" localSheetId="2" hidden="1">Planilha2!$D$4:$D$520</definedName>
+    <definedName name="_ECO_RANGE_ID803c298d378e4e53a4a20af695306fa8" localSheetId="2" hidden="1">Planilha2!$P$4:$P$520</definedName>
+    <definedName name="_ECO_RANGE_ID8079f7254e2045d7b6f108b6090661af" localSheetId="2" hidden="1">Planilha2!$K$4:$K$520</definedName>
+    <definedName name="_ECO_RANGE_ID8258752d88ae4a28954d28ad5fcf6494" localSheetId="0" hidden="1">Plan1!$K$4:$K$520</definedName>
+    <definedName name="_ECO_RANGE_ID82d0a60c3afb42b19d6637d0b52de21b" localSheetId="1" hidden="1">Planilha1!$B$3</definedName>
+    <definedName name="_ECO_RANGE_ID8a1e3cf1e7b74535a905ef94e4d254c9" localSheetId="1" hidden="1">Planilha1!$E$4:$E$520</definedName>
+    <definedName name="_ECO_RANGE_ID8c1d5e3844834eeebcfe00230f782c77" localSheetId="0" hidden="1">Plan1!$B$3</definedName>
+    <definedName name="_ECO_RANGE_ID8e814f8fbfb04b8b8b9162949b217602" localSheetId="2" hidden="1">Planilha2!$J$4:$J$520</definedName>
+    <definedName name="_ECO_RANGE_ID94a1b39ace404d86aea765cca07b7768" localSheetId="1" hidden="1">Planilha1!$G$4:$G$520</definedName>
+    <definedName name="_ECO_RANGE_ID98daf1eea7984e309160618397c42286" localSheetId="0" hidden="1">Plan1!$L$4:$L$520</definedName>
+    <definedName name="_ECO_RANGE_IDa1e78211d505468a8b4fc2f73bb90796" localSheetId="1" hidden="1">Planilha1!$M$4:$M$520</definedName>
+    <definedName name="_ECO_RANGE_IDb4a33ad0c3d34222a89e48026c852975" localSheetId="2" hidden="1">Planilha2!$G$4:$G$520</definedName>
+    <definedName name="_ECO_RANGE_IDbc6b6810878c4635b6969e8333e36e15" localSheetId="0" hidden="1">Plan1!$D$4:$D$520</definedName>
+    <definedName name="_ECO_RANGE_IDbcd0637b3bac483ea32e81fdf9367b27" localSheetId="1" hidden="1">Planilha1!$I$4:$I$520</definedName>
+    <definedName name="_ECO_RANGE_IDbd90a3a88d744777af77b45a06210090" localSheetId="0" hidden="1">Plan1!$F$4:$F$520</definedName>
+    <definedName name="_ECO_RANGE_IDcb3baf54ce74467f9d1716d99ff648f1" localSheetId="2" hidden="1">Planilha2!$O$4:$O$520</definedName>
+    <definedName name="_ECO_RANGE_IDdafb3dbd943f4032911c13aa7d6be3c2" localSheetId="0" hidden="1">Plan1!$H$4:$H$520</definedName>
+    <definedName name="_ECO_RANGE_IDe2df1625c8a14d449bde8d5eb2bea39d" localSheetId="0" hidden="1">Plan1!$N$4:$N$520</definedName>
+    <definedName name="_ECO_RANGE_IDe870ce9738e44447abf55ea8cb0e828c" localSheetId="2" hidden="1">Planilha2!$C$4:$C$520</definedName>
+    <definedName name="_ECO_RANGE_IDebbf75e0e68747e9870eb91d5c806d1e" localSheetId="0" hidden="1">Plan1!$O$4:$O$520</definedName>
+    <definedName name="_ECO_RANGE_IDec6caad9a63840cabcca4e9e1d54c8df" localSheetId="1" hidden="1">Planilha1!$F$4:$F$520</definedName>
+    <definedName name="_ECO_RANGE_IDede280d4f0454684b338ce5bcbefcad4" localSheetId="0" hidden="1">Plan1!$M$4:$M$520</definedName>
+    <definedName name="_ECO_RANGE_IDf3786d2b6653470bad140a5a96cab8aa" localSheetId="1" hidden="1">Planilha1!$L$4:$L$520</definedName>
+    <definedName name="_ECO_RANGE_IDf57cdd634e5e4bf08f4c46d2ed3a87a7" localSheetId="1" hidden="1">Planilha1!$H$4:$H$520</definedName>
+    <definedName name="_ECO_RANGE_IDf6d9829051de4f5a94a1ebde127e6f0c" localSheetId="2" hidden="1">Planilha2!$E$4:$E$520</definedName>
+    <definedName name="_ECO_RANGE_IDfa710064f2ba4e4a9b558aa31df35ba8" localSheetId="1" hidden="1">Planilha1!$A$4:$B$520</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -284,300 +284,306 @@
 <file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
       <tp>
         <v>3</v>
         <stp/>
-        <stp>651e0012-4377-47a7-bd8e-2053c1351fc1</stp>
+        <stp>0bdcb314-7246-4ef8-89c3-23688f1dd90c</stp>
+        <tr r="N3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>44fbb5ac-5081-462e-b4b0-fb723145c3c2</stp>
+        <tr r="H3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>f0936590-4cb4-4e5d-bd47-514885d13796</stp>
+        <tr r="H3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>e4d3a1a4-4412-43d0-9af1-6c28c0d60a5f</stp>
+        <tr r="L3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>cc843460-5eb2-47a1-8bc9-6430ed87a4dd</stp>
+        <tr r="E3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>7f51c7e4-5873-47ec-b10c-815adfa30788</stp>
+        <tr r="N3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>bce5bb52-c764-4ff1-ae21-b4440543f71b</stp>
+        <tr r="M3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>395aa6eb-d304-494d-baa0-973bf65608fc</stp>
+        <tr r="K3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>271089d8-0f89-4d82-8c7c-35f031201f1a</stp>
+        <tr r="F3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>f0503939-e635-4631-b91c-1f9cf7b98fc8</stp>
+        <tr r="I3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>d63ec3be-56bd-4a23-8b7d-72b3a8deee7e</stp>
+        <tr r="D3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>4fb53643-9ff0-4bc5-a4a0-2aa3c22d0484</stp>
+        <tr r="A3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>aac1fb66-59d7-430e-94d9-04295f27f8e6</stp>
+        <tr r="L3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>d66f48d3-e41e-4a23-a8d5-4af8f0f5512c</stp>
+        <tr r="F3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>257e0c77-bcb1-4f90-92bf-d80321f7a325</stp>
+        <tr r="F3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>7938d4e6-a46d-471a-965c-8be763bd764f</stp>
+        <tr r="E3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>97002e4f-1ab1-47d0-b375-32cf48acc02a</stp>
+        <tr r="J3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>30c84831-0915-4125-9148-a8315a629a90</stp>
+        <tr r="D3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>d8d1787e-b94e-48e7-bccf-92eaffb5ecaf</stp>
+        <tr r="M3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a75a1e91-c552-4712-b736-bf54f235de08</stp>
+        <tr r="J3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>fabba9e5-1a1b-4af8-a8e1-1f9553ba6b19</stp>
+        <tr r="K3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>78d838cf-5050-4a84-8a76-1f932a788234</stp>
+        <tr r="M3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>b72d3b00-f148-42af-a557-57fcc1c07d5b</stp>
+        <tr r="G3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>9d24ebec-5e55-4f91-8f62-3bd0d6fc8ee7</stp>
+        <tr r="J3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>ef730f98-94a7-4c69-a945-0e572c1fc704</stp>
+        <tr r="P3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>0ca6638d-9227-4ce5-b929-110b6cf9c952</stp>
+        <tr r="O3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>aae2c522-7090-407f-9011-bca5a26efbfc</stp>
+        <tr r="K3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>e6a2c5a6-08fd-4b0a-9fd9-429b02ed31fc</stp>
+        <tr r="L3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>c0bdaad9-3857-417a-acf0-481fc958abc2</stp>
+        <tr r="G3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>146f523e-2569-48cd-abb1-5578b7fd9634</stp>
+        <tr r="C3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a3b2a6b5-f4f8-4cab-9d6b-1b4dbac4f2a0</stp>
+        <tr r="G3" s="3"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>7703c5cb-2d32-4c50-ab20-1a0a8e403068</stp>
+        <tr r="A3" s="2"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a6223661-5fa1-4c9d-a998-b6396d3ff310</stp>
+        <tr r="I3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>ee885619-11bd-447a-b1b5-775c881a2e6a</stp>
+        <tr r="N3" s="2"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>d1038500-a6e1-42d0-ad92-409080660acf</stp>
+        <tr r="A3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a7c9ff5d-16e8-43fa-9c8c-5c3641f0cf19</stp>
+        <tr r="H3" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>07a938b9-6beb-4bad-9aea-d20e0577d287</stp>
+        <tr r="E3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>389450e8-1548-4792-a07c-6964004e389b</stp>
+        <tr r="D3" s="1"/>
+      </tp>
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>292ad6d9-608e-4494-926c-17a9beafce21</stp>
+        <tr r="O3" s="3"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_eco_9bbdf10e619f4d8fb0becfb7c6ebd3a9">
+      <tp>
+        <v>3</v>
+        <stp/>
+        <stp>a6f1019d-c3ac-4005-917a-e5f459514e3b</stp>
         <tr r="O3" s="2"/>
       </tp>
       <tp>
         <v>3</v>
         <stp/>
-        <stp>5c284fe6-32ce-4540-9e0b-b8dfeb18055b</stp>
+        <stp>53d2961b-51d5-4cf1-a405-c973ca96df6e</stp>
         <tr r="I3" s="3"/>
       </tp>
       <tp>
         <v>3</v>
         <stp/>
-        <stp>0fae79ac-b820-4bef-bbcd-e60ae439ec0a</stp>
-        <tr r="F3" s="1"/>
+        <stp>758bee03-f8d4-4cb9-a022-ba5ba1168b0d</stp>
+        <tr r="C3" s="1"/>
       </tp>
       <tp>
         <v>3</v>
         <stp/>
-        <stp>b141a3b4-55d4-4bde-a394-c076c3fbe012</stp>
-        <tr r="H3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>8f5fba8f-79ad-4e6b-999a-44c71b05de57</stp>
+        <stp>6b236d58-efc5-4209-a6d2-afd3fd4ab31c</stp>
         <tr r="C3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>a2251b01-aedc-4289-aa18-14afd4015a39</stp>
-        <tr r="H3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>83bcbf2c-ab75-4fde-b420-08aa99a7b80a</stp>
-        <tr r="F3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>34ed34ea-4bea-411b-806a-992e1275463b</stp>
-        <tr r="E3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>aa60246a-c683-4068-b6ff-f4a05b633be6</stp>
-        <tr r="E3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>3b76ab7a-d3ac-4c52-87e5-b8f44a56d691</stp>
-        <tr r="L3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>612ef0ab-c5a9-4644-8c16-bea17d5da981</stp>
-        <tr r="A3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>5a276a4e-a38b-4ea7-8a95-5ca0fe80c6c3</stp>
-        <tr r="F3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>6ba51716-09d3-402a-9998-daf254bb370f</stp>
-        <tr r="C3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>0ce85a8e-5771-4ebf-83a3-49eec1a13fd0</stp>
-        <tr r="K3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>40fb259b-7203-4902-ae09-e0e7283e1fa0</stp>
-        <tr r="K3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>a06e5785-eae8-4cd1-8428-0aaedbadc337</stp>
-        <tr r="G3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>6bf6d21a-a716-4e10-bd45-b46aea434136</stp>
-        <tr r="M3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>2ac33508-667b-42d5-ac3a-16c530cf73a7</stp>
-        <tr r="D3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>9a829019-f63f-4980-a213-d1b97ef15204</stp>
-        <tr r="D3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>4a14c25a-c931-410f-ab82-7313393ee44b</stp>
-        <tr r="M3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>09141432-6a45-4e29-91c2-d2809d270ded</stp>
-        <tr r="C3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>cf48377e-438f-4f4d-b3d9-3aa155539b53</stp>
-        <tr r="A3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>6aa58b9c-5de2-4307-ac19-61a0350c5ffd</stp>
-        <tr r="L3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>71862d1f-1374-431a-8907-d2c83f1c93d7</stp>
-        <tr r="M3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>1e0f62dc-a1b4-4ce5-a9ac-efb12ba313ba</stp>
-        <tr r="H3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>bb586066-c948-457d-bbdc-5a93e06ec477</stp>
-        <tr r="N3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>e998bcf1-d070-44b4-bbd2-f812f46204ac</stp>
-        <tr r="N3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>f2cd3e29-b279-4188-936c-10caa4e5b67f</stp>
-        <tr r="K3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>a9db0880-6629-4e1d-848d-c167f5cb4fd7</stp>
-        <tr r="G3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>7c8665e3-0701-46db-a91d-76e6635ef941</stp>
-        <tr r="D3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>2997b43d-a6ac-4fcc-a4ff-a3d4ec9a423e</stp>
-        <tr r="L3" s="2"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>f1fb2c7a-646a-439c-ad4d-e904c23c53a4</stp>
-        <tr r="A3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>e85303c7-4450-4411-87a5-6f5b6f0b6eb0</stp>
-        <tr r="E3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>4c0b1ccd-b2cd-4ccd-a922-2a4f1a2c194e</stp>
-        <tr r="J3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>97aaf7e5-f754-43e9-94e9-62ad665aa1a0</stp>
-        <tr r="N3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>92bb70ff-4e9e-4457-9ad7-924b8e6e60ca</stp>
-        <tr r="G3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>ea97e4ec-9e47-43be-9392-5e57d3e4cdbb</stp>
-        <tr r="I3" s="2"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>c62f33e1-bb3c-40e5-a564-6ef9fe0c6aed</stp>
-        <tr r="O3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>1f63dc19-d7ea-4680-840b-1f9c8cec5a77</stp>
-        <tr r="O3" s="1"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>99089bdc-7689-4349-b886-e8fecde4044b</stp>
-        <tr r="J3" s="3"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>7d8fb1cc-613d-4f1e-b66b-c2d8771ae156</stp>
-        <tr r="I3" s="1"/>
-      </tp>
-    </main>
-    <main first="rtdsrv_eco_50809abfbf9147b480bf275a66dbf246">
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>4118678b-6a94-4506-931e-9495ac877f90</stp>
-        <tr r="P3" s="3"/>
-      </tp>
-      <tp>
-        <v>3</v>
-        <stp/>
-        <stp>3fd1c9b3-4cf8-4aab-9f4b-39c2877875c2</stp>
-        <tr r="J3" s="2"/>
       </tp>
     </main>
   </volType>
@@ -847,7 +853,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O511"/>
+  <dimension ref="A1:O520"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -23441,6 +23447,363 @@
         <v>7.0507999999999997</v>
       </c>
     </row>
+    <row r="512" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A512" s="1">
+        <v>46122</v>
+      </c>
+      <c r="C512">
+        <v>8.7428000000000008</v>
+      </c>
+      <c r="D512">
+        <v>7.8758999999999997</v>
+      </c>
+      <c r="E512">
+        <v>7.7671000000000001</v>
+      </c>
+      <c r="F512">
+        <v>7.7013999999999996</v>
+      </c>
+      <c r="G512">
+        <v>7.7309999999999999</v>
+      </c>
+      <c r="H512">
+        <v>7.6281999999999996</v>
+      </c>
+      <c r="I512">
+        <v>7.6009000000000002</v>
+      </c>
+      <c r="J512">
+        <v>7.45</v>
+      </c>
+      <c r="K512">
+        <v>7.2171000000000003</v>
+      </c>
+      <c r="L512">
+        <v>7.1083999999999996</v>
+      </c>
+      <c r="M512">
+        <v>7.0396999999999998</v>
+      </c>
+      <c r="N512">
+        <v>7.0155000000000003</v>
+      </c>
+      <c r="O512">
+        <v>6.9955999999999996</v>
+      </c>
+    </row>
+    <row r="513" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A513" s="1">
+        <v>46125</v>
+      </c>
+      <c r="C513">
+        <v>8.5763999999999996</v>
+      </c>
+      <c r="D513">
+        <v>7.8589000000000002</v>
+      </c>
+      <c r="E513">
+        <v>7.7241</v>
+      </c>
+      <c r="F513">
+        <v>7.65</v>
+      </c>
+      <c r="G513">
+        <v>7.67</v>
+      </c>
+      <c r="H513">
+        <v>7.5655999999999999</v>
+      </c>
+      <c r="I513">
+        <v>7.54</v>
+      </c>
+      <c r="J513">
+        <v>7.4</v>
+      </c>
+      <c r="K513">
+        <v>7.1807999999999996</v>
+      </c>
+      <c r="L513">
+        <v>7.0848000000000004</v>
+      </c>
+      <c r="M513">
+        <v>7.0210999999999997</v>
+      </c>
+      <c r="N513">
+        <v>7</v>
+      </c>
+      <c r="O513">
+        <v>6.9848999999999997</v>
+      </c>
+    </row>
+    <row r="514" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A514" s="1">
+        <v>46126</v>
+      </c>
+      <c r="C514">
+        <v>8.6949000000000005</v>
+      </c>
+      <c r="D514">
+        <v>7.8410000000000002</v>
+      </c>
+      <c r="E514">
+        <v>7.69</v>
+      </c>
+      <c r="F514">
+        <v>7.6102999999999996</v>
+      </c>
+      <c r="G514">
+        <v>7.6402999999999999</v>
+      </c>
+      <c r="H514">
+        <v>7.5339999999999998</v>
+      </c>
+      <c r="I514">
+        <v>7.5046999999999997</v>
+      </c>
+      <c r="J514">
+        <v>7.37</v>
+      </c>
+      <c r="K514">
+        <v>7.17</v>
+      </c>
+      <c r="L514">
+        <v>7.0835999999999997</v>
+      </c>
+      <c r="M514">
+        <v>7.0202</v>
+      </c>
+      <c r="N514">
+        <v>7.0083000000000002</v>
+      </c>
+      <c r="O514">
+        <v>6.9922000000000004</v>
+      </c>
+    </row>
+    <row r="515" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A515" s="1">
+        <v>46127</v>
+      </c>
+      <c r="C515">
+        <v>8.6300000000000008</v>
+      </c>
+      <c r="D515">
+        <v>7.8029999999999999</v>
+      </c>
+      <c r="E515">
+        <v>7.68</v>
+      </c>
+      <c r="F515">
+        <v>7.58</v>
+      </c>
+      <c r="G515">
+        <v>7.62</v>
+      </c>
+      <c r="H515">
+        <v>7.5301999999999998</v>
+      </c>
+      <c r="I515">
+        <v>7.4950999999999999</v>
+      </c>
+      <c r="J515">
+        <v>7.3699000000000003</v>
+      </c>
+      <c r="K515">
+        <v>7.17</v>
+      </c>
+      <c r="L515">
+        <v>7.0914000000000001</v>
+      </c>
+      <c r="M515">
+        <v>7.0201000000000002</v>
+      </c>
+      <c r="N515">
+        <v>7.0069999999999997</v>
+      </c>
+      <c r="O515">
+        <v>6.9954000000000001</v>
+      </c>
+    </row>
+    <row r="516" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A516" s="1">
+        <v>46128</v>
+      </c>
+      <c r="C516">
+        <v>8.7057000000000002</v>
+      </c>
+      <c r="D516">
+        <v>7.85</v>
+      </c>
+      <c r="E516">
+        <v>7.7462</v>
+      </c>
+      <c r="F516">
+        <v>7.6375000000000002</v>
+      </c>
+      <c r="G516">
+        <v>7.66</v>
+      </c>
+      <c r="H516">
+        <v>7.5484999999999998</v>
+      </c>
+      <c r="I516">
+        <v>7.5155000000000003</v>
+      </c>
+      <c r="J516">
+        <v>7.3849999999999998</v>
+      </c>
+      <c r="K516">
+        <v>7.1658999999999997</v>
+      </c>
+      <c r="L516">
+        <v>7.0884999999999998</v>
+      </c>
+      <c r="M516">
+        <v>7.02</v>
+      </c>
+      <c r="N516">
+        <v>7.0077999999999996</v>
+      </c>
+      <c r="O516">
+        <v>6.9973000000000001</v>
+      </c>
+    </row>
+    <row r="517" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A517" s="1">
+        <v>46129</v>
+      </c>
+      <c r="C517">
+        <v>8.9298000000000002</v>
+      </c>
+      <c r="D517">
+        <v>7.8986999999999998</v>
+      </c>
+      <c r="E517">
+        <v>7.7365000000000004</v>
+      </c>
+      <c r="F517">
+        <v>7.6159999999999997</v>
+      </c>
+      <c r="G517">
+        <v>7.63</v>
+      </c>
+      <c r="H517">
+        <v>7.51</v>
+      </c>
+      <c r="I517">
+        <v>7.4844999999999997</v>
+      </c>
+      <c r="J517">
+        <v>7.36</v>
+      </c>
+      <c r="K517">
+        <v>7.15</v>
+      </c>
+      <c r="L517">
+        <v>7.0754999999999999</v>
+      </c>
+      <c r="M517">
+        <v>7.0110000000000001</v>
+      </c>
+      <c r="N517">
+        <v>7.0141</v>
+      </c>
+      <c r="O517">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="518" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A518" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C518">
+        <v>8.8671000000000006</v>
+      </c>
+      <c r="D518">
+        <v>7.9</v>
+      </c>
+      <c r="E518">
+        <v>7.7286999999999999</v>
+      </c>
+      <c r="F518">
+        <v>7.61</v>
+      </c>
+      <c r="G518">
+        <v>7.6173999999999999</v>
+      </c>
+      <c r="H518">
+        <v>7.4832000000000001</v>
+      </c>
+      <c r="I518">
+        <v>7.4577999999999998</v>
+      </c>
+      <c r="J518">
+        <v>7.3319999999999999</v>
+      </c>
+      <c r="K518">
+        <v>7.1220999999999997</v>
+      </c>
+      <c r="L518">
+        <v>7.06</v>
+      </c>
+      <c r="M518">
+        <v>6.9962</v>
+      </c>
+      <c r="N518">
+        <v>6.9928999999999997</v>
+      </c>
+      <c r="O518">
+        <v>6.98</v>
+      </c>
+    </row>
+    <row r="519" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A519" s="1">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="520" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A520" s="1">
+        <v>46134</v>
+      </c>
+      <c r="C520">
+        <v>8.7578999999999994</v>
+      </c>
+      <c r="D520">
+        <v>7.9194000000000004</v>
+      </c>
+      <c r="E520">
+        <v>7.77</v>
+      </c>
+      <c r="F520">
+        <v>7.6627999999999998</v>
+      </c>
+      <c r="G520">
+        <v>7.6707999999999998</v>
+      </c>
+      <c r="H520">
+        <v>7.5397999999999996</v>
+      </c>
+      <c r="I520">
+        <v>7.5198</v>
+      </c>
+      <c r="J520">
+        <v>7.38</v>
+      </c>
+      <c r="K520">
+        <v>7.16</v>
+      </c>
+      <c r="L520">
+        <v>7.0877999999999997</v>
+      </c>
+      <c r="M520">
+        <v>7.0366</v>
+      </c>
+      <c r="N520">
+        <v>7.0339</v>
+      </c>
+      <c r="O520">
+        <v>7.03</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -23448,7 +23811,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2426C424-F8DA-489F-86D1-16CF91ECBA06}">
-  <dimension ref="A1:O511"/>
+  <dimension ref="A1:O520"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -46042,6 +46405,363 @@
         <v>4104.5295260000003</v>
       </c>
     </row>
+    <row r="512" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A512" s="1">
+        <v>46122</v>
+      </c>
+      <c r="C512">
+        <v>4666.778824</v>
+      </c>
+      <c r="D512">
+        <v>4695.4273800000001</v>
+      </c>
+      <c r="E512">
+        <v>4544.9267790000004</v>
+      </c>
+      <c r="F512">
+        <v>4579.7083110000003</v>
+      </c>
+      <c r="G512">
+        <v>4434.9486230000002</v>
+      </c>
+      <c r="H512">
+        <v>4353.3109729999996</v>
+      </c>
+      <c r="I512">
+        <v>4397.5766800000001</v>
+      </c>
+      <c r="J512">
+        <v>4363.9993400000003</v>
+      </c>
+      <c r="K512">
+        <v>4235.2348620000002</v>
+      </c>
+      <c r="L512">
+        <v>4274.805155</v>
+      </c>
+      <c r="M512">
+        <v>4181.0649149999999</v>
+      </c>
+      <c r="N512">
+        <v>4228.6911550000004</v>
+      </c>
+      <c r="O512">
+        <v>4142.1060520000001</v>
+      </c>
+    </row>
+    <row r="513" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A513" s="1">
+        <v>46125</v>
+      </c>
+      <c r="C513">
+        <v>4672.7512219999999</v>
+      </c>
+      <c r="D513">
+        <v>4699.5673370000004</v>
+      </c>
+      <c r="E513">
+        <v>4552.1417410000004</v>
+      </c>
+      <c r="F513">
+        <v>4589.0249889999996</v>
+      </c>
+      <c r="G513">
+        <v>4447.697572</v>
+      </c>
+      <c r="H513">
+        <v>4369.7286560000002</v>
+      </c>
+      <c r="I513">
+        <v>4414.7879469999998</v>
+      </c>
+      <c r="J513">
+        <v>4380.9631280000003</v>
+      </c>
+      <c r="K513">
+        <v>4251.7433529999998</v>
+      </c>
+      <c r="L513">
+        <v>4288.0102459999998</v>
+      </c>
+      <c r="M513">
+        <v>4192.9047909999999</v>
+      </c>
+      <c r="N513">
+        <v>4239.50497</v>
+      </c>
+      <c r="O513">
+        <v>4150.6377750000001</v>
+      </c>
+    </row>
+    <row r="514" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A514" s="1">
+        <v>46126</v>
+      </c>
+      <c r="C514">
+        <v>4674.4862450000001</v>
+      </c>
+      <c r="D514">
+        <v>4703.7426290000003</v>
+      </c>
+      <c r="E514">
+        <v>4558.5397819999998</v>
+      </c>
+      <c r="F514">
+        <v>4596.970609</v>
+      </c>
+      <c r="G514">
+        <v>4455.5328330000002</v>
+      </c>
+      <c r="H514">
+        <v>4379.5680700000003</v>
+      </c>
+      <c r="I514">
+        <v>4426.1036109999995</v>
+      </c>
+      <c r="J514">
+        <v>4392.4001449999996</v>
+      </c>
+      <c r="K514">
+        <v>4258.7400930000003</v>
+      </c>
+      <c r="L514">
+        <v>4291.4859409999999</v>
+      </c>
+      <c r="M514">
+        <v>4196.2193450000004</v>
+      </c>
+      <c r="N514">
+        <v>4238.1723359999996</v>
+      </c>
+      <c r="O514">
+        <v>4149.5950489999996</v>
+      </c>
+    </row>
+    <row r="515" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A515" s="1">
+        <v>46127</v>
+      </c>
+      <c r="C515">
+        <v>4678.9277179999999</v>
+      </c>
+      <c r="D515">
+        <v>4708.8225270000003</v>
+      </c>
+      <c r="E515">
+        <v>4562.7038819999998</v>
+      </c>
+      <c r="F515">
+        <v>4603.8004810000002</v>
+      </c>
+      <c r="G515">
+        <v>4461.8924379999999</v>
+      </c>
+      <c r="H515">
+        <v>4383.4705560000002</v>
+      </c>
+      <c r="I515">
+        <v>4431.4555319999999</v>
+      </c>
+      <c r="J515">
+        <v>4395.4995129999998</v>
+      </c>
+      <c r="K515">
+        <v>4261.6902200000004</v>
+      </c>
+      <c r="L515">
+        <v>4291.0476040000003</v>
+      </c>
+      <c r="M515">
+        <v>4199.1480570000003</v>
+      </c>
+      <c r="N515">
+        <v>4241.7447700000002</v>
+      </c>
+      <c r="O515">
+        <v>4150.7378140000001</v>
+      </c>
+    </row>
+    <row r="516" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A516" s="1">
+        <v>46128</v>
+      </c>
+      <c r="C516">
+        <v>4680.9622220000001</v>
+      </c>
+      <c r="D516">
+        <v>4709.721826</v>
+      </c>
+      <c r="E516">
+        <v>4559.4912260000001</v>
+      </c>
+      <c r="F516">
+        <v>4599.9192270000003</v>
+      </c>
+      <c r="G516">
+        <v>4458.4118749999998</v>
+      </c>
+      <c r="H516">
+        <v>4382.3101839999999</v>
+      </c>
+      <c r="I516">
+        <v>4429.4839760000004</v>
+      </c>
+      <c r="J516">
+        <v>4394.0159789999998</v>
+      </c>
+      <c r="K516">
+        <v>4265.8459400000002</v>
+      </c>
+      <c r="L516">
+        <v>4294.9327839999996</v>
+      </c>
+      <c r="M516">
+        <v>4201.7492339999999</v>
+      </c>
+      <c r="N516">
+        <v>4243.9116000000004</v>
+      </c>
+      <c r="O516">
+        <v>4152.2520469999999</v>
+      </c>
+    </row>
+    <row r="517" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A517" s="1">
+        <v>46129</v>
+      </c>
+      <c r="C517">
+        <v>4680.9259119999997</v>
+      </c>
+      <c r="D517">
+        <v>4710.5604020000001</v>
+      </c>
+      <c r="E517">
+        <v>4563.2811510000001</v>
+      </c>
+      <c r="F517">
+        <v>4605.3549240000002</v>
+      </c>
+      <c r="G517">
+        <v>4465.9460929999996</v>
+      </c>
+      <c r="H517">
+        <v>4393.2931930000004</v>
+      </c>
+      <c r="I517">
+        <v>4439.4681890000002</v>
+      </c>
+      <c r="J517">
+        <v>4403.7309679999998</v>
+      </c>
+      <c r="K517">
+        <v>4274.441914</v>
+      </c>
+      <c r="L517">
+        <v>4303.2252950000002</v>
+      </c>
+      <c r="M517">
+        <v>4208.6633549999997</v>
+      </c>
+      <c r="N517">
+        <v>4243.2782349999998</v>
+      </c>
+      <c r="O517">
+        <v>4153.3365999999996</v>
+      </c>
+    </row>
+    <row r="518" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A518" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C518">
+        <v>4684.9776199999997</v>
+      </c>
+      <c r="D518">
+        <v>4713.5181430000002</v>
+      </c>
+      <c r="E518">
+        <v>4566.8906790000001</v>
+      </c>
+      <c r="F518">
+        <v>4608.9646769999999</v>
+      </c>
+      <c r="G518">
+        <v>4470.7482710000004</v>
+      </c>
+      <c r="H518">
+        <v>4401.7850859999999</v>
+      </c>
+      <c r="I518">
+        <v>4448.4669219999996</v>
+      </c>
+      <c r="J518">
+        <v>4414.3034340000004</v>
+      </c>
+      <c r="K518">
+        <v>4287.5855700000002</v>
+      </c>
+      <c r="L518">
+        <v>4312.6269430000002</v>
+      </c>
+      <c r="M518">
+        <v>4218.397841</v>
+      </c>
+      <c r="N518">
+        <v>4256.7013649999999</v>
+      </c>
+      <c r="O518">
+        <v>4166.5187390000001</v>
+      </c>
+    </row>
+    <row r="519" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A519" s="1">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="520" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A520" s="1">
+        <v>46134</v>
+      </c>
+      <c r="C520">
+        <v>4689.6585999999998</v>
+      </c>
+      <c r="D520">
+        <v>4715.6818149999999</v>
+      </c>
+      <c r="E520">
+        <v>4566.00036</v>
+      </c>
+      <c r="F520">
+        <v>4605.664589</v>
+      </c>
+      <c r="G520">
+        <v>4465.1738539999997</v>
+      </c>
+      <c r="H520">
+        <v>4392.4295840000004</v>
+      </c>
+      <c r="I520">
+        <v>4436.8155210000004</v>
+      </c>
+      <c r="J520">
+        <v>4403.6138099999998</v>
+      </c>
+      <c r="K520">
+        <v>4275.9217619999999</v>
+      </c>
+      <c r="L520">
+        <v>4303.1101959999996</v>
+      </c>
+      <c r="M520">
+        <v>4201.403926</v>
+      </c>
+      <c r="N520">
+        <v>4238.3493109999999</v>
+      </c>
+      <c r="O520">
+        <v>4142.478494</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -46049,7 +46769,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE81DAD-ED15-4633-A0F7-1D8C32328F6D}">
-  <dimension ref="A1:Z511"/>
+  <dimension ref="A1:Z520"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -68602,6 +69322,363 @@
         <v>9.2999999999999999E-2</v>
       </c>
     </row>
+    <row r="512" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A512" s="1">
+        <v>46122</v>
+      </c>
+      <c r="D512">
+        <v>-6.8999999999999999E-3</v>
+      </c>
+      <c r="E512">
+        <v>7.1000000000000004E-3</v>
+      </c>
+      <c r="F512">
+        <v>8.6999999999999994E-3</v>
+      </c>
+      <c r="G512">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="H512">
+        <v>2.53E-2</v>
+      </c>
+      <c r="I512">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="J512">
+        <v>5.3600000000000002E-2</v>
+      </c>
+      <c r="K512">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="L512">
+        <v>6.7299999999999999E-2</v>
+      </c>
+      <c r="M512">
+        <v>7.3300000000000004E-2</v>
+      </c>
+      <c r="N512">
+        <v>7.3800000000000004E-2</v>
+      </c>
+      <c r="O512">
+        <v>8.5699999999999998E-2</v>
+      </c>
+      <c r="P512">
+        <v>9.0999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="513" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A513" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D513">
+        <v>-4.7999999999999996E-3</v>
+      </c>
+      <c r="E513">
+        <v>8.6999999999999994E-3</v>
+      </c>
+      <c r="F513">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="G513">
+        <v>1.5100000000000001E-2</v>
+      </c>
+      <c r="H513">
+        <v>2.52E-2</v>
+      </c>
+      <c r="I513">
+        <v>4.1200000000000001E-2</v>
+      </c>
+      <c r="J513">
+        <v>5.3600000000000002E-2</v>
+      </c>
+      <c r="K513">
+        <v>6.4199999999999993E-2</v>
+      </c>
+      <c r="L513">
+        <v>6.7299999999999999E-2</v>
+      </c>
+      <c r="M513">
+        <v>7.3300000000000004E-2</v>
+      </c>
+      <c r="N513">
+        <v>7.3800000000000004E-2</v>
+      </c>
+      <c r="O513">
+        <v>8.5800000000000001E-2</v>
+      </c>
+      <c r="P513">
+        <v>9.0800000000000006E-2</v>
+      </c>
+    </row>
+    <row r="514" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A514" s="1">
+        <v>46126</v>
+      </c>
+      <c r="D514">
+        <v>-2.8E-3</v>
+      </c>
+      <c r="E514">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="F514">
+        <v>1.17E-2</v>
+      </c>
+      <c r="G514">
+        <v>1.55E-2</v>
+      </c>
+      <c r="H514">
+        <v>2.5499999999999998E-2</v>
+      </c>
+      <c r="I514">
+        <v>4.1500000000000002E-2</v>
+      </c>
+      <c r="J514">
+        <v>5.3699999999999998E-2</v>
+      </c>
+      <c r="K514">
+        <v>6.4299999999999996E-2</v>
+      </c>
+      <c r="L514">
+        <v>6.7599999999999993E-2</v>
+      </c>
+      <c r="M514">
+        <v>7.3499999999999996E-2</v>
+      </c>
+      <c r="N514">
+        <v>7.3899999999999993E-2</v>
+      </c>
+      <c r="O514">
+        <v>8.5699999999999998E-2</v>
+      </c>
+      <c r="P514">
+        <v>9.06E-2</v>
+      </c>
+    </row>
+    <row r="515" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A515" s="1">
+        <v>46127</v>
+      </c>
+      <c r="D515">
+        <v>-1.6000000000000001E-3</v>
+      </c>
+      <c r="E515">
+        <v>1.0800000000000001E-2</v>
+      </c>
+      <c r="F515">
+        <v>1.2200000000000001E-2</v>
+      </c>
+      <c r="G515">
+        <v>1.5699999999999999E-2</v>
+      </c>
+      <c r="H515">
+        <v>2.6100000000000002E-2</v>
+      </c>
+      <c r="I515">
+        <v>4.2500000000000003E-2</v>
+      </c>
+      <c r="J515">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="K515">
+        <v>6.6400000000000001E-2</v>
+      </c>
+      <c r="L515">
+        <v>6.8500000000000005E-2</v>
+      </c>
+      <c r="M515">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="N515">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="O515">
+        <v>8.5599999999999996E-2</v>
+      </c>
+      <c r="P515">
+        <v>9.06E-2</v>
+      </c>
+    </row>
+    <row r="516" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A516" s="1">
+        <v>46128</v>
+      </c>
+      <c r="D516">
+        <v>-8.0000000000000004E-4</v>
+      </c>
+      <c r="E516">
+        <v>1.0800000000000001E-2</v>
+      </c>
+      <c r="F516">
+        <v>1.2800000000000001E-2</v>
+      </c>
+      <c r="G516">
+        <v>1.66E-2</v>
+      </c>
+      <c r="H516">
+        <v>2.69E-2</v>
+      </c>
+      <c r="I516">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="J516">
+        <v>5.5399999999999998E-2</v>
+      </c>
+      <c r="K516">
+        <v>6.7699999999999996E-2</v>
+      </c>
+      <c r="L516">
+        <v>7.1499999999999994E-2</v>
+      </c>
+      <c r="M516">
+        <v>7.5499999999999998E-2</v>
+      </c>
+      <c r="N516">
+        <v>7.51E-2</v>
+      </c>
+      <c r="O516">
+        <v>8.5500000000000007E-2</v>
+      </c>
+      <c r="P516">
+        <v>9.06E-2</v>
+      </c>
+    </row>
+    <row r="517" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A517" s="1">
+        <v>46129</v>
+      </c>
+      <c r="D517">
+        <v>-5.9999999999999995E-4</v>
+      </c>
+      <c r="E517">
+        <v>1.03E-2</v>
+      </c>
+      <c r="F517">
+        <v>1.3599999999999999E-2</v>
+      </c>
+      <c r="G517">
+        <v>1.6799999999999999E-2</v>
+      </c>
+      <c r="H517">
+        <v>2.7099999999999999E-2</v>
+      </c>
+      <c r="I517">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="J517">
+        <v>5.5500000000000001E-2</v>
+      </c>
+      <c r="K517">
+        <v>6.7900000000000002E-2</v>
+      </c>
+      <c r="L517">
+        <v>7.1900000000000006E-2</v>
+      </c>
+      <c r="M517">
+        <v>7.5499999999999998E-2</v>
+      </c>
+      <c r="N517">
+        <v>7.5499999999999998E-2</v>
+      </c>
+      <c r="O517">
+        <v>8.5500000000000007E-2</v>
+      </c>
+      <c r="P517">
+        <v>9.0499999999999997E-2</v>
+      </c>
+    </row>
+    <row r="518" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A518" s="1">
+        <v>46132</v>
+      </c>
+      <c r="D518">
+        <v>-5.9999999999999995E-4</v>
+      </c>
+      <c r="E518">
+        <v>9.9000000000000008E-3</v>
+      </c>
+      <c r="F518">
+        <v>1.34E-2</v>
+      </c>
+      <c r="G518">
+        <v>1.6899999999999998E-2</v>
+      </c>
+      <c r="H518">
+        <v>2.7300000000000001E-2</v>
+      </c>
+      <c r="I518">
+        <v>4.4200000000000003E-2</v>
+      </c>
+      <c r="J518">
+        <v>5.5800000000000002E-2</v>
+      </c>
+      <c r="K518">
+        <v>6.7900000000000002E-2</v>
+      </c>
+      <c r="L518">
+        <v>7.2099999999999997E-2</v>
+      </c>
+      <c r="M518">
+        <v>7.5499999999999998E-2</v>
+      </c>
+      <c r="N518">
+        <v>7.5399999999999995E-2</v>
+      </c>
+      <c r="O518">
+        <v>8.4900000000000003E-2</v>
+      </c>
+      <c r="P518">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="519" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A519" s="1">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="520" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A520" s="1">
+        <v>46134</v>
+      </c>
+      <c r="D520">
+        <v>-2.3999999999999998E-3</v>
+      </c>
+      <c r="E520">
+        <v>8.8000000000000005E-3</v>
+      </c>
+      <c r="F520">
+        <v>1.3100000000000001E-2</v>
+      </c>
+      <c r="G520">
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="H520">
+        <v>2.7300000000000001E-2</v>
+      </c>
+      <c r="I520">
+        <v>4.4499999999999998E-2</v>
+      </c>
+      <c r="J520">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="K520">
+        <v>6.83E-2</v>
+      </c>
+      <c r="L520">
+        <v>7.2599999999999998E-2</v>
+      </c>
+      <c r="M520">
+        <v>7.5600000000000001E-2</v>
+      </c>
+      <c r="N520">
+        <v>7.5399999999999995E-2</v>
+      </c>
+      <c r="O520">
+        <v>8.4599999999999995E-2</v>
+      </c>
+      <c r="P520">
+        <v>8.9599999999999999E-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>